<commit_message>
Progress on Form 4MB
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-3DA.xlsx
+++ b/form_reporting_templates/Form-3DA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data_dissemination\iotc-reference-forms\form_reporting_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF33E15-70C0-4DDA-B641-119C42F3BDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A37B023-2FAC-4CE1-8DA5-43A5567EFFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="5DvQh67CqwpXF5nvK7dpPxR3Pt0yB/nZxqejbtUHEzmemyWSbLakjzpL/AJnjHY2PfyZeKC6tZsl2wcqhenc9Q==" workbookSaltValue="SFs4XJpRzZAAYXRJrz5n4w==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{742ED9EC-8AD9-42B2-9B99-191B35B67816}"/>
@@ -1144,6 +1144,24 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1153,15 +1171,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1169,15 +1178,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2324,35 +2324,35 @@
       <c r="E4" s="122"/>
       <c r="F4" s="122"/>
       <c r="G4" s="123"/>
-      <c r="H4" s="124" t="s">
+      <c r="H4" s="130" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="125"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="126"/>
+      <c r="I4" s="131"/>
+      <c r="J4" s="131"/>
+      <c r="K4" s="132"/>
       <c r="L4" s="121" t="s">
         <v>50</v>
       </c>
       <c r="M4" s="122"/>
       <c r="N4" s="123"/>
-      <c r="O4" s="124" t="s">
+      <c r="O4" s="130" t="s">
         <v>28</v>
       </c>
-      <c r="P4" s="125"/>
-      <c r="Q4" s="125"/>
-      <c r="R4" s="125"/>
-      <c r="S4" s="125"/>
-      <c r="T4" s="125"/>
-      <c r="U4" s="126"/>
-      <c r="V4" s="124" t="s">
+      <c r="P4" s="131"/>
+      <c r="Q4" s="131"/>
+      <c r="R4" s="131"/>
+      <c r="S4" s="131"/>
+      <c r="T4" s="131"/>
+      <c r="U4" s="132"/>
+      <c r="V4" s="130" t="s">
         <v>29</v>
       </c>
-      <c r="W4" s="125"/>
-      <c r="X4" s="125"/>
-      <c r="Y4" s="125"/>
-      <c r="Z4" s="125"/>
-      <c r="AA4" s="125"/>
-      <c r="AB4" s="126"/>
+      <c r="W4" s="131"/>
+      <c r="X4" s="131"/>
+      <c r="Y4" s="131"/>
+      <c r="Z4" s="131"/>
+      <c r="AA4" s="131"/>
+      <c r="AB4" s="132"/>
       <c r="AC4" s="98" t="s">
         <v>31</v>
       </c>
@@ -2458,33 +2458,33 @@
       <c r="DY4" s="75"/>
     </row>
     <row r="5" spans="2:129" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="127"/>
-      <c r="C5" s="128"/>
-      <c r="D5" s="128"/>
-      <c r="E5" s="128"/>
-      <c r="F5" s="128"/>
-      <c r="G5" s="129"/>
-      <c r="H5" s="130"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="131"/>
-      <c r="K5" s="132"/>
-      <c r="L5" s="127"/>
-      <c r="M5" s="128"/>
-      <c r="N5" s="129"/>
-      <c r="O5" s="130"/>
-      <c r="P5" s="131"/>
-      <c r="Q5" s="131"/>
-      <c r="R5" s="131"/>
-      <c r="S5" s="131"/>
-      <c r="T5" s="131"/>
-      <c r="U5" s="132"/>
-      <c r="V5" s="130"/>
-      <c r="W5" s="131"/>
-      <c r="X5" s="131"/>
-      <c r="Y5" s="131"/>
-      <c r="Z5" s="131"/>
-      <c r="AA5" s="131"/>
-      <c r="AB5" s="132"/>
+      <c r="B5" s="124"/>
+      <c r="C5" s="125"/>
+      <c r="D5" s="125"/>
+      <c r="E5" s="125"/>
+      <c r="F5" s="125"/>
+      <c r="G5" s="126"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="134"/>
+      <c r="J5" s="134"/>
+      <c r="K5" s="135"/>
+      <c r="L5" s="124"/>
+      <c r="M5" s="125"/>
+      <c r="N5" s="126"/>
+      <c r="O5" s="133"/>
+      <c r="P5" s="134"/>
+      <c r="Q5" s="134"/>
+      <c r="R5" s="134"/>
+      <c r="S5" s="134"/>
+      <c r="T5" s="134"/>
+      <c r="U5" s="135"/>
+      <c r="V5" s="133"/>
+      <c r="W5" s="134"/>
+      <c r="X5" s="134"/>
+      <c r="Y5" s="134"/>
+      <c r="Z5" s="134"/>
+      <c r="AA5" s="134"/>
+      <c r="AB5" s="135"/>
       <c r="AC5" s="99" t="s">
         <v>34</v>
       </c>
@@ -2590,19 +2590,19 @@
       <c r="DY5" s="78"/>
     </row>
     <row r="6" spans="2:129" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="133"/>
-      <c r="C6" s="134"/>
-      <c r="D6" s="134"/>
-      <c r="E6" s="134"/>
-      <c r="F6" s="134"/>
-      <c r="G6" s="135"/>
+      <c r="B6" s="127"/>
+      <c r="C6" s="128"/>
+      <c r="D6" s="128"/>
+      <c r="E6" s="128"/>
+      <c r="F6" s="128"/>
+      <c r="G6" s="129"/>
       <c r="H6" s="136"/>
       <c r="I6" s="137"/>
       <c r="J6" s="137"/>
       <c r="K6" s="138"/>
-      <c r="L6" s="133"/>
-      <c r="M6" s="134"/>
-      <c r="N6" s="135"/>
+      <c r="L6" s="127"/>
+      <c r="M6" s="128"/>
+      <c r="N6" s="129"/>
       <c r="O6" s="136"/>
       <c r="P6" s="137"/>
       <c r="Q6" s="137"/>
@@ -4459,7 +4459,8 @@
       <c r="AB57" s="66"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="wikyZqsXjk/9IO9lE8aGull6Pg4nypopq0WLt/g5N8liPDMJtCccgZbxulSxu06CUSQuUBf+psDgjTd8bcgsrw==" saltValue="QZw6ftz9lx6RQXYlsU0zNg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="XoJ5qKY8Y7diJeHOoqSg7/iXi7jVb2oZrNE3shpeeCqp4ZpWVDoC4maZ75Vu8I/xZdIwwFAlwW1C84unNxDyDg==" saltValue="B9Z2aag2RkRnYzQWHF1+rg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <dataConsolidate/>
   <mergeCells count="7">
     <mergeCell ref="AD3:DY3"/>
     <mergeCell ref="B2:AB3"/>
@@ -4480,7 +4481,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC4:AC7 M7:N7 K7" xr:uid="{86B40B65-30E0-465F-9E4E-BDD2D0A3ECB3}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC4:AC7 L7 K7 B7 C7 D7 E7 F7 G7 H7 I7 J7 N7 M7" xr:uid="{86B40B65-30E0-465F-9E4E-BDD2D0A3ECB3}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Addition of month into 3DA form - removed from reporting metadata
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-3DA.xlsx
+++ b/form_reporting_templates/Form-3DA.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A37B023-2FAC-4CE1-8DA5-43A5567EFFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92877180-9F71-4BDD-8E01-FEA27F862130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="5DvQh67CqwpXF5nvK7dpPxR3Pt0yB/nZxqejbtUHEzmemyWSbLakjzpL/AJnjHY2PfyZeKC6tZsl2wcqhenc9Q==" workbookSaltValue="SFs4XJpRzZAAYXRJrz5n4w==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{742ED9EC-8AD9-42B2-9B99-191B35B67816}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{742ED9EC-8AD9-42B2-9B99-191B35B67816}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -81,9 +81,6 @@
     <t>Reporting entity</t>
   </si>
   <si>
-    <t>Reporting month</t>
-  </si>
-  <si>
     <t>Vessel name</t>
   </si>
   <si>
@@ -190,6 +187,9 @@
   </si>
   <si>
     <t>DFOB</t>
+  </si>
+  <si>
+    <t>Month</t>
   </si>
 </sst>
 </file>
@@ -771,7 +771,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1071,12 +1071,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1187,6 +1181,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1532,44 +1529,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC2D41B5-AC8B-4133-9C08-EAF515BF72F5}">
   <dimension ref="B1:H32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="2.85546875" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
-    <col min="6" max="6" width="27.140625" customWidth="1"/>
-    <col min="7" max="7" width="28.5703125" customWidth="1"/>
-    <col min="8" max="8" width="2.85546875" customWidth="1"/>
+    <col min="1" max="2" width="2.88671875" customWidth="1"/>
+    <col min="3" max="3" width="27.109375" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" customWidth="1"/>
+    <col min="7" max="7" width="28.5546875" customWidth="1"/>
+    <col min="8" max="8" width="2.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="110" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-      <c r="E2" s="111"/>
-      <c r="F2" s="111"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="112"/>
-    </row>
-    <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="113"/>
-      <c r="C3" s="114"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="114"/>
-      <c r="F3" s="114"/>
-      <c r="G3" s="114"/>
-      <c r="H3" s="115"/>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B2" s="108" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="110"/>
+    </row>
+    <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="111"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="112"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="113"/>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" s="31"/>
       <c r="C4" s="32" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E4" s="34"/>
       <c r="F4" s="32" t="s">
@@ -1580,7 +1577,7 @@
       </c>
       <c r="H4" s="36"/>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="20"/>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
@@ -1589,7 +1586,7 @@
       <c r="G5" s="23"/>
       <c r="H5" s="19"/>
     </row>
-    <row r="6" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B6" s="20"/>
       <c r="C6" s="27" t="s">
         <v>7</v>
@@ -1600,7 +1597,7 @@
       <c r="G6" s="23"/>
       <c r="H6" s="19"/>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="20"/>
       <c r="C7" s="23"/>
       <c r="D7" s="23"/>
@@ -1609,20 +1606,20 @@
       <c r="G7" s="23"/>
       <c r="H7" s="19"/>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="20"/>
-      <c r="C8" s="109" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="109"/>
+      <c r="C8" s="107" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="107"/>
       <c r="E8" s="23"/>
-      <c r="F8" s="109" t="s">
+      <c r="F8" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="G8" s="109"/>
+      <c r="G8" s="107"/>
       <c r="H8" s="19"/>
     </row>
-    <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="20"/>
       <c r="C9" s="30" t="s">
         <v>1</v>
@@ -1635,20 +1632,20 @@
       <c r="G9" s="3"/>
       <c r="H9" s="19"/>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="20"/>
       <c r="C10" s="21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="23"/>
       <c r="F10" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="19"/>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="D11" s="22"/>
@@ -1657,29 +1654,29 @@
       <c r="G11" s="22"/>
       <c r="H11" s="19"/>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="20"/>
       <c r="C12" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="105"/>
+        <v>40</v>
+      </c>
+      <c r="D12" s="103"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
       <c r="G12" s="23"/>
       <c r="H12" s="19"/>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="20"/>
       <c r="C13" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="105"/>
+      <c r="D13" s="103"/>
       <c r="E13" s="23"/>
       <c r="F13" s="23"/>
       <c r="G13" s="23"/>
       <c r="H13" s="19"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" s="20"/>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
@@ -1688,7 +1685,7 @@
       <c r="G14" s="23"/>
       <c r="H14" s="19"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="20"/>
       <c r="C15" s="26"/>
       <c r="D15" s="26"/>
@@ -1697,7 +1694,7 @@
       <c r="G15" s="26"/>
       <c r="H15" s="19"/>
     </row>
-    <row r="16" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B16" s="20"/>
       <c r="C16" s="27" t="s">
         <v>3</v>
@@ -1708,7 +1705,7 @@
       <c r="G16" s="23"/>
       <c r="H16" s="19"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="20"/>
       <c r="C17" s="23"/>
       <c r="D17" s="23"/>
@@ -1717,20 +1714,18 @@
       <c r="G17" s="23"/>
       <c r="H17" s="19"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="20"/>
       <c r="C18" s="21" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="23"/>
-      <c r="F18" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" s="4"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="23"/>
       <c r="H18" s="19"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="20"/>
       <c r="C19" s="28" t="s">
         <v>13</v>
@@ -1741,10 +1736,10 @@
       <c r="G19" s="23"/>
       <c r="H19" s="19"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="20"/>
       <c r="C20" s="28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="23"/>
@@ -1752,7 +1747,7 @@
       <c r="G20" s="23"/>
       <c r="H20" s="19"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="20"/>
       <c r="C21" s="21"/>
       <c r="D21" s="22"/>
@@ -1761,7 +1756,7 @@
       <c r="G21" s="23"/>
       <c r="H21" s="19"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22" s="20"/>
       <c r="C22" s="26"/>
       <c r="D22" s="25"/>
@@ -1770,7 +1765,7 @@
       <c r="G22" s="26"/>
       <c r="H22" s="19"/>
     </row>
-    <row r="23" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B23" s="20"/>
       <c r="C23" s="27" t="s">
         <v>5</v>
@@ -1781,7 +1776,7 @@
       <c r="G23" s="23"/>
       <c r="H23" s="19"/>
     </row>
-    <row r="24" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="20"/>
       <c r="C24" s="27"/>
       <c r="D24" s="22"/>
@@ -1790,20 +1785,20 @@
       <c r="G24" s="23"/>
       <c r="H24" s="19"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B25" s="20"/>
       <c r="C25" s="28" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="97" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E25" s="23"/>
       <c r="F25" s="23"/>
       <c r="G25" s="23"/>
       <c r="H25" s="19"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B26" s="20"/>
       <c r="C26" s="21"/>
       <c r="D26" s="22"/>
@@ -1812,7 +1807,7 @@
       <c r="G26" s="23"/>
       <c r="H26" s="19"/>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B27" s="20"/>
       <c r="C27" s="24"/>
       <c r="D27" s="25"/>
@@ -1821,7 +1816,7 @@
       <c r="G27" s="26"/>
       <c r="H27" s="19"/>
     </row>
-    <row r="28" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="18" x14ac:dyDescent="0.35">
       <c r="B28" s="20"/>
       <c r="C28" s="27" t="s">
         <v>6</v>
@@ -1832,7 +1827,7 @@
       <c r="G28" s="23"/>
       <c r="H28" s="19"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B29" s="20"/>
       <c r="C29" s="23"/>
       <c r="D29" s="23"/>
@@ -1841,16 +1836,16 @@
       <c r="G29" s="23"/>
       <c r="H29" s="19"/>
     </row>
-    <row r="30" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="20"/>
-      <c r="C30" s="106"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="107"/>
-      <c r="F30" s="107"/>
-      <c r="G30" s="108"/>
+      <c r="C30" s="104"/>
+      <c r="D30" s="105"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="106"/>
       <c r="H30" s="19"/>
     </row>
-    <row r="31" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="16"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -1859,12 +1854,12 @@
       <c r="G31" s="17"/>
       <c r="H31" s="18"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
       <c r="C32" s="1"/>
       <c r="D32" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="Nh1s6ywUuHHMLTLqcrCD1BhG1EDYi+sM8o47yMg2bNl+HZTOE3MnCBbUaim6mTQCChNRnpJYi1QozsuxLiqLzQ==" saltValue="LH2dbLUnt4lNORYa+jABeA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="8zgQK6CzseY/nXEsmcZ6KOc2LPjCqDpvMhKJ0fDGq3Ki7c6VfA7bpvVqJONHNXpvQ0DZ9wEG8vX+A7WZW59XTQ==" saltValue="1JDIDjt1WL8b3miAPASWbQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="4">
     <mergeCell ref="C30:G30"/>
     <mergeCell ref="C8:D8"/>
@@ -1888,68 +1883,69 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C098252-FABC-4161-882E-794F98E79BC6}">
-  <dimension ref="B1:DY57"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:DZ57"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" style="92" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="92" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" style="96" customWidth="1"/>
-    <col min="6" max="6" width="17.140625" style="12" customWidth="1"/>
-    <col min="7" max="7" width="17.140625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" style="47" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.140625" style="51" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" style="49" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" style="50" customWidth="1"/>
-    <col min="12" max="12" width="17.140625" style="51" customWidth="1"/>
-    <col min="13" max="13" width="10" style="49" customWidth="1"/>
-    <col min="14" max="14" width="10" style="50" customWidth="1"/>
-    <col min="15" max="15" width="7.140625" style="47" customWidth="1"/>
-    <col min="16" max="16" width="7.140625" style="49" customWidth="1"/>
-    <col min="17" max="19" width="7.85546875" style="58" customWidth="1"/>
-    <col min="20" max="20" width="7.140625" style="49" customWidth="1"/>
-    <col min="21" max="21" width="10" style="55" customWidth="1"/>
-    <col min="22" max="22" width="7.140625" style="51" customWidth="1"/>
-    <col min="23" max="23" width="7.140625" style="49" customWidth="1"/>
-    <col min="24" max="26" width="7.85546875" style="58" customWidth="1"/>
-    <col min="27" max="27" width="7.140625" style="49" customWidth="1"/>
-    <col min="28" max="28" width="10" style="67" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" style="72" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="9.140625" style="85"/>
-    <col min="31" max="128" width="9.140625" style="86"/>
-    <col min="129" max="129" width="9.140625" style="87"/>
+    <col min="1" max="1" width="2.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" style="92" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" style="92" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="92" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" style="96" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" style="12" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" style="10" customWidth="1"/>
+    <col min="9" max="9" width="7.88671875" style="47" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.109375" style="51" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" style="49" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="50" customWidth="1"/>
+    <col min="13" max="13" width="17.109375" style="51" customWidth="1"/>
+    <col min="14" max="14" width="10" style="49" customWidth="1"/>
+    <col min="15" max="15" width="10" style="50" customWidth="1"/>
+    <col min="16" max="16" width="7.109375" style="47" customWidth="1"/>
+    <col min="17" max="17" width="7.109375" style="49" customWidth="1"/>
+    <col min="18" max="20" width="7.88671875" style="58" customWidth="1"/>
+    <col min="21" max="21" width="7.109375" style="49" customWidth="1"/>
+    <col min="22" max="22" width="10" style="55" customWidth="1"/>
+    <col min="23" max="23" width="7.109375" style="51" customWidth="1"/>
+    <col min="24" max="24" width="7.109375" style="49" customWidth="1"/>
+    <col min="25" max="27" width="7.88671875" style="58" customWidth="1"/>
+    <col min="28" max="28" width="7.109375" style="49" customWidth="1"/>
+    <col min="29" max="29" width="10" style="67" customWidth="1"/>
+    <col min="30" max="30" width="11.5546875" style="72" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.109375" style="85"/>
+    <col min="32" max="129" width="9.109375" style="86"/>
+    <col min="130" max="130" width="9.109375" style="87"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:129" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:130" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="8"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="93"/>
       <c r="G1" s="8"/>
-      <c r="H1" s="46"/>
+      <c r="H1" s="8"/>
       <c r="I1" s="46"/>
-      <c r="J1" s="48"/>
+      <c r="J1" s="46"/>
       <c r="K1" s="48"/>
       <c r="L1" s="48"/>
       <c r="M1" s="48"/>
       <c r="N1" s="48"/>
       <c r="O1" s="48"/>
       <c r="P1" s="48"/>
-      <c r="Q1" s="52"/>
+      <c r="Q1" s="48"/>
       <c r="R1" s="52"/>
       <c r="S1" s="52"/>
-      <c r="T1" s="48"/>
-      <c r="U1" s="52"/>
-      <c r="V1" s="48"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="48"/>
+      <c r="V1" s="52"/>
       <c r="W1" s="48"/>
-      <c r="X1" s="52"/>
+      <c r="X1" s="48"/>
       <c r="Y1" s="52"/>
       <c r="Z1" s="52"/>
-      <c r="AA1" s="48"/>
-      <c r="AB1" s="52"/>
-      <c r="AC1"/>
+      <c r="AA1" s="52"/>
+      <c r="AB1" s="48"/>
+      <c r="AC1" s="52"/>
       <c r="AD1"/>
       <c r="AE1"/>
       <c r="AF1"/>
@@ -2050,38 +2046,39 @@
       <c r="DW1"/>
       <c r="DX1"/>
       <c r="DY1"/>
-    </row>
-    <row r="2" spans="2:129" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="110" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-      <c r="E2" s="111"/>
-      <c r="F2" s="111"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="111"/>
-      <c r="I2" s="111"/>
-      <c r="J2" s="111"/>
-      <c r="K2" s="111"/>
-      <c r="L2" s="111"/>
-      <c r="M2" s="111"/>
-      <c r="N2" s="111"/>
-      <c r="O2" s="111"/>
-      <c r="P2" s="111"/>
-      <c r="Q2" s="111"/>
-      <c r="R2" s="111"/>
-      <c r="S2" s="111"/>
-      <c r="T2" s="111"/>
-      <c r="U2" s="111"/>
-      <c r="V2" s="111"/>
-      <c r="W2" s="111"/>
-      <c r="X2" s="111"/>
-      <c r="Y2" s="111"/>
-      <c r="Z2" s="111"/>
-      <c r="AA2" s="111"/>
-      <c r="AB2" s="111"/>
-      <c r="AC2" s="68"/>
+      <c r="DZ1"/>
+    </row>
+    <row r="2" spans="2:130" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="108" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="109"/>
+      <c r="M2" s="109"/>
+      <c r="N2" s="109"/>
+      <c r="O2" s="109"/>
+      <c r="P2" s="109"/>
+      <c r="Q2" s="109"/>
+      <c r="R2" s="109"/>
+      <c r="S2" s="109"/>
+      <c r="T2" s="109"/>
+      <c r="U2" s="109"/>
+      <c r="V2" s="109"/>
+      <c r="W2" s="109"/>
+      <c r="X2" s="109"/>
+      <c r="Y2" s="109"/>
+      <c r="Z2" s="109"/>
+      <c r="AA2" s="109"/>
+      <c r="AB2" s="109"/>
+      <c r="AC2" s="109"/>
       <c r="AD2" s="68"/>
       <c r="AE2" s="68"/>
       <c r="AF2" s="68"/>
@@ -2181,183 +2178,185 @@
       <c r="DV2" s="68"/>
       <c r="DW2" s="68"/>
       <c r="DX2" s="68"/>
-      <c r="DY2" s="69"/>
-    </row>
-    <row r="3" spans="2:129" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="119"/>
-      <c r="C3" s="120"/>
-      <c r="D3" s="120"/>
-      <c r="E3" s="120"/>
-      <c r="F3" s="120"/>
-      <c r="G3" s="120"/>
-      <c r="H3" s="120"/>
-      <c r="I3" s="120"/>
-      <c r="J3" s="120"/>
-      <c r="K3" s="120"/>
-      <c r="L3" s="120"/>
-      <c r="M3" s="120"/>
-      <c r="N3" s="120"/>
-      <c r="O3" s="120"/>
-      <c r="P3" s="120"/>
-      <c r="Q3" s="120"/>
-      <c r="R3" s="120"/>
-      <c r="S3" s="120"/>
-      <c r="T3" s="120"/>
-      <c r="U3" s="120"/>
-      <c r="V3" s="120"/>
-      <c r="W3" s="120"/>
-      <c r="X3" s="120"/>
-      <c r="Y3" s="120"/>
-      <c r="Z3" s="120"/>
-      <c r="AA3" s="120"/>
-      <c r="AB3" s="120"/>
-      <c r="AC3" s="70"/>
-      <c r="AD3" s="116" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE3" s="117"/>
-      <c r="AF3" s="117"/>
-      <c r="AG3" s="117"/>
-      <c r="AH3" s="117"/>
-      <c r="AI3" s="117"/>
-      <c r="AJ3" s="117"/>
-      <c r="AK3" s="117"/>
-      <c r="AL3" s="117"/>
-      <c r="AM3" s="117"/>
-      <c r="AN3" s="117"/>
-      <c r="AO3" s="117"/>
-      <c r="AP3" s="117"/>
-      <c r="AQ3" s="117"/>
-      <c r="AR3" s="117"/>
-      <c r="AS3" s="117"/>
-      <c r="AT3" s="117"/>
-      <c r="AU3" s="117"/>
-      <c r="AV3" s="117"/>
-      <c r="AW3" s="117"/>
-      <c r="AX3" s="117"/>
-      <c r="AY3" s="117"/>
-      <c r="AZ3" s="117"/>
-      <c r="BA3" s="117"/>
-      <c r="BB3" s="117"/>
-      <c r="BC3" s="117"/>
-      <c r="BD3" s="117"/>
-      <c r="BE3" s="117"/>
-      <c r="BF3" s="117"/>
-      <c r="BG3" s="117"/>
-      <c r="BH3" s="117"/>
-      <c r="BI3" s="117"/>
-      <c r="BJ3" s="117"/>
-      <c r="BK3" s="117"/>
-      <c r="BL3" s="117"/>
-      <c r="BM3" s="117"/>
-      <c r="BN3" s="117"/>
-      <c r="BO3" s="117"/>
-      <c r="BP3" s="117"/>
-      <c r="BQ3" s="117"/>
-      <c r="BR3" s="117"/>
-      <c r="BS3" s="117"/>
-      <c r="BT3" s="117"/>
-      <c r="BU3" s="117"/>
-      <c r="BV3" s="117"/>
-      <c r="BW3" s="117"/>
-      <c r="BX3" s="117"/>
-      <c r="BY3" s="117"/>
-      <c r="BZ3" s="117"/>
-      <c r="CA3" s="117"/>
-      <c r="CB3" s="117"/>
-      <c r="CC3" s="117"/>
-      <c r="CD3" s="117"/>
-      <c r="CE3" s="117"/>
-      <c r="CF3" s="117"/>
-      <c r="CG3" s="117"/>
-      <c r="CH3" s="117"/>
-      <c r="CI3" s="117"/>
-      <c r="CJ3" s="117"/>
-      <c r="CK3" s="117"/>
-      <c r="CL3" s="117"/>
-      <c r="CM3" s="117"/>
-      <c r="CN3" s="117"/>
-      <c r="CO3" s="117"/>
-      <c r="CP3" s="117"/>
-      <c r="CQ3" s="117"/>
-      <c r="CR3" s="117"/>
-      <c r="CS3" s="117"/>
-      <c r="CT3" s="117"/>
-      <c r="CU3" s="117"/>
-      <c r="CV3" s="117"/>
-      <c r="CW3" s="117"/>
-      <c r="CX3" s="117"/>
-      <c r="CY3" s="117"/>
-      <c r="CZ3" s="117"/>
-      <c r="DA3" s="117"/>
-      <c r="DB3" s="117"/>
-      <c r="DC3" s="117"/>
-      <c r="DD3" s="117"/>
-      <c r="DE3" s="117"/>
-      <c r="DF3" s="117"/>
-      <c r="DG3" s="117"/>
-      <c r="DH3" s="117"/>
-      <c r="DI3" s="117"/>
-      <c r="DJ3" s="117"/>
-      <c r="DK3" s="117"/>
-      <c r="DL3" s="117"/>
-      <c r="DM3" s="117"/>
-      <c r="DN3" s="117"/>
-      <c r="DO3" s="117"/>
-      <c r="DP3" s="117"/>
-      <c r="DQ3" s="117"/>
-      <c r="DR3" s="117"/>
-      <c r="DS3" s="117"/>
-      <c r="DT3" s="117"/>
-      <c r="DU3" s="117"/>
-      <c r="DV3" s="117"/>
-      <c r="DW3" s="117"/>
-      <c r="DX3" s="117"/>
-      <c r="DY3" s="118"/>
-    </row>
-    <row r="4" spans="2:129" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="121" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="122"/>
-      <c r="D4" s="122"/>
-      <c r="E4" s="122"/>
-      <c r="F4" s="122"/>
-      <c r="G4" s="123"/>
-      <c r="H4" s="130" t="s">
+      <c r="DY2" s="68"/>
+      <c r="DZ2" s="69"/>
+    </row>
+    <row r="3" spans="2:130" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="117"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="118"/>
+      <c r="E3" s="118"/>
+      <c r="F3" s="118"/>
+      <c r="G3" s="118"/>
+      <c r="H3" s="118"/>
+      <c r="I3" s="118"/>
+      <c r="J3" s="118"/>
+      <c r="K3" s="118"/>
+      <c r="L3" s="118"/>
+      <c r="M3" s="118"/>
+      <c r="N3" s="118"/>
+      <c r="O3" s="118"/>
+      <c r="P3" s="118"/>
+      <c r="Q3" s="118"/>
+      <c r="R3" s="118"/>
+      <c r="S3" s="118"/>
+      <c r="T3" s="118"/>
+      <c r="U3" s="118"/>
+      <c r="V3" s="118"/>
+      <c r="W3" s="118"/>
+      <c r="X3" s="118"/>
+      <c r="Y3" s="118"/>
+      <c r="Z3" s="118"/>
+      <c r="AA3" s="118"/>
+      <c r="AB3" s="118"/>
+      <c r="AC3" s="118"/>
+      <c r="AD3" s="70"/>
+      <c r="AE3" s="114" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF3" s="115"/>
+      <c r="AG3" s="115"/>
+      <c r="AH3" s="115"/>
+      <c r="AI3" s="115"/>
+      <c r="AJ3" s="115"/>
+      <c r="AK3" s="115"/>
+      <c r="AL3" s="115"/>
+      <c r="AM3" s="115"/>
+      <c r="AN3" s="115"/>
+      <c r="AO3" s="115"/>
+      <c r="AP3" s="115"/>
+      <c r="AQ3" s="115"/>
+      <c r="AR3" s="115"/>
+      <c r="AS3" s="115"/>
+      <c r="AT3" s="115"/>
+      <c r="AU3" s="115"/>
+      <c r="AV3" s="115"/>
+      <c r="AW3" s="115"/>
+      <c r="AX3" s="115"/>
+      <c r="AY3" s="115"/>
+      <c r="AZ3" s="115"/>
+      <c r="BA3" s="115"/>
+      <c r="BB3" s="115"/>
+      <c r="BC3" s="115"/>
+      <c r="BD3" s="115"/>
+      <c r="BE3" s="115"/>
+      <c r="BF3" s="115"/>
+      <c r="BG3" s="115"/>
+      <c r="BH3" s="115"/>
+      <c r="BI3" s="115"/>
+      <c r="BJ3" s="115"/>
+      <c r="BK3" s="115"/>
+      <c r="BL3" s="115"/>
+      <c r="BM3" s="115"/>
+      <c r="BN3" s="115"/>
+      <c r="BO3" s="115"/>
+      <c r="BP3" s="115"/>
+      <c r="BQ3" s="115"/>
+      <c r="BR3" s="115"/>
+      <c r="BS3" s="115"/>
+      <c r="BT3" s="115"/>
+      <c r="BU3" s="115"/>
+      <c r="BV3" s="115"/>
+      <c r="BW3" s="115"/>
+      <c r="BX3" s="115"/>
+      <c r="BY3" s="115"/>
+      <c r="BZ3" s="115"/>
+      <c r="CA3" s="115"/>
+      <c r="CB3" s="115"/>
+      <c r="CC3" s="115"/>
+      <c r="CD3" s="115"/>
+      <c r="CE3" s="115"/>
+      <c r="CF3" s="115"/>
+      <c r="CG3" s="115"/>
+      <c r="CH3" s="115"/>
+      <c r="CI3" s="115"/>
+      <c r="CJ3" s="115"/>
+      <c r="CK3" s="115"/>
+      <c r="CL3" s="115"/>
+      <c r="CM3" s="115"/>
+      <c r="CN3" s="115"/>
+      <c r="CO3" s="115"/>
+      <c r="CP3" s="115"/>
+      <c r="CQ3" s="115"/>
+      <c r="CR3" s="115"/>
+      <c r="CS3" s="115"/>
+      <c r="CT3" s="115"/>
+      <c r="CU3" s="115"/>
+      <c r="CV3" s="115"/>
+      <c r="CW3" s="115"/>
+      <c r="CX3" s="115"/>
+      <c r="CY3" s="115"/>
+      <c r="CZ3" s="115"/>
+      <c r="DA3" s="115"/>
+      <c r="DB3" s="115"/>
+      <c r="DC3" s="115"/>
+      <c r="DD3" s="115"/>
+      <c r="DE3" s="115"/>
+      <c r="DF3" s="115"/>
+      <c r="DG3" s="115"/>
+      <c r="DH3" s="115"/>
+      <c r="DI3" s="115"/>
+      <c r="DJ3" s="115"/>
+      <c r="DK3" s="115"/>
+      <c r="DL3" s="115"/>
+      <c r="DM3" s="115"/>
+      <c r="DN3" s="115"/>
+      <c r="DO3" s="115"/>
+      <c r="DP3" s="115"/>
+      <c r="DQ3" s="115"/>
+      <c r="DR3" s="115"/>
+      <c r="DS3" s="115"/>
+      <c r="DT3" s="115"/>
+      <c r="DU3" s="115"/>
+      <c r="DV3" s="115"/>
+      <c r="DW3" s="115"/>
+      <c r="DX3" s="115"/>
+      <c r="DY3" s="115"/>
+      <c r="DZ3" s="116"/>
+    </row>
+    <row r="4" spans="2:130" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="119" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="120"/>
+      <c r="D4" s="120"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="120"/>
+      <c r="G4" s="120"/>
+      <c r="H4" s="121"/>
+      <c r="I4" s="128" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="129"/>
+      <c r="K4" s="129"/>
+      <c r="L4" s="130"/>
+      <c r="M4" s="119" t="s">
+        <v>49</v>
+      </c>
+      <c r="N4" s="120"/>
+      <c r="O4" s="121"/>
+      <c r="P4" s="128" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="131"/>
-      <c r="J4" s="131"/>
-      <c r="K4" s="132"/>
-      <c r="L4" s="121" t="s">
-        <v>50</v>
-      </c>
-      <c r="M4" s="122"/>
-      <c r="N4" s="123"/>
-      <c r="O4" s="130" t="s">
+      <c r="Q4" s="129"/>
+      <c r="R4" s="129"/>
+      <c r="S4" s="129"/>
+      <c r="T4" s="129"/>
+      <c r="U4" s="129"/>
+      <c r="V4" s="130"/>
+      <c r="W4" s="128" t="s">
         <v>28</v>
       </c>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
-      <c r="R4" s="131"/>
-      <c r="S4" s="131"/>
-      <c r="T4" s="131"/>
-      <c r="U4" s="132"/>
-      <c r="V4" s="130" t="s">
-        <v>29</v>
-      </c>
-      <c r="W4" s="131"/>
-      <c r="X4" s="131"/>
-      <c r="Y4" s="131"/>
-      <c r="Z4" s="131"/>
-      <c r="AA4" s="131"/>
-      <c r="AB4" s="132"/>
-      <c r="AC4" s="98" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD4" s="73"/>
-      <c r="AE4" s="74"/>
+      <c r="X4" s="129"/>
+      <c r="Y4" s="129"/>
+      <c r="Z4" s="129"/>
+      <c r="AA4" s="129"/>
+      <c r="AB4" s="129"/>
+      <c r="AC4" s="130"/>
+      <c r="AD4" s="98" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE4" s="73"/>
       <c r="AF4" s="74"/>
       <c r="AG4" s="74"/>
       <c r="AH4" s="74"/>
@@ -2455,41 +2454,42 @@
       <c r="DV4" s="74"/>
       <c r="DW4" s="74"/>
       <c r="DX4" s="74"/>
-      <c r="DY4" s="75"/>
-    </row>
-    <row r="5" spans="2:129" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="124"/>
-      <c r="C5" s="125"/>
-      <c r="D5" s="125"/>
-      <c r="E5" s="125"/>
-      <c r="F5" s="125"/>
-      <c r="G5" s="126"/>
-      <c r="H5" s="133"/>
-      <c r="I5" s="134"/>
-      <c r="J5" s="134"/>
-      <c r="K5" s="135"/>
-      <c r="L5" s="124"/>
-      <c r="M5" s="125"/>
-      <c r="N5" s="126"/>
-      <c r="O5" s="133"/>
-      <c r="P5" s="134"/>
-      <c r="Q5" s="134"/>
-      <c r="R5" s="134"/>
-      <c r="S5" s="134"/>
-      <c r="T5" s="134"/>
-      <c r="U5" s="135"/>
+      <c r="DY4" s="74"/>
+      <c r="DZ4" s="75"/>
+    </row>
+    <row r="5" spans="2:130" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="122"/>
+      <c r="C5" s="137"/>
+      <c r="D5" s="137"/>
+      <c r="E5" s="137"/>
+      <c r="F5" s="137"/>
+      <c r="G5" s="137"/>
+      <c r="H5" s="124"/>
+      <c r="I5" s="131"/>
+      <c r="J5" s="132"/>
+      <c r="K5" s="132"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="122"/>
+      <c r="N5" s="123"/>
+      <c r="O5" s="124"/>
+      <c r="P5" s="131"/>
+      <c r="Q5" s="132"/>
+      <c r="R5" s="132"/>
+      <c r="S5" s="132"/>
+      <c r="T5" s="132"/>
+      <c r="U5" s="132"/>
       <c r="V5" s="133"/>
-      <c r="W5" s="134"/>
-      <c r="X5" s="134"/>
-      <c r="Y5" s="134"/>
-      <c r="Z5" s="134"/>
-      <c r="AA5" s="134"/>
-      <c r="AB5" s="135"/>
-      <c r="AC5" s="99" t="s">
-        <v>34</v>
-      </c>
-      <c r="AD5" s="76"/>
-      <c r="AE5" s="77"/>
+      <c r="W5" s="131"/>
+      <c r="X5" s="132"/>
+      <c r="Y5" s="132"/>
+      <c r="Z5" s="132"/>
+      <c r="AA5" s="132"/>
+      <c r="AB5" s="132"/>
+      <c r="AC5" s="133"/>
+      <c r="AD5" s="99" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE5" s="76"/>
       <c r="AF5" s="77"/>
       <c r="AG5" s="77"/>
       <c r="AH5" s="77"/>
@@ -2587,41 +2587,42 @@
       <c r="DV5" s="77"/>
       <c r="DW5" s="77"/>
       <c r="DX5" s="77"/>
-      <c r="DY5" s="78"/>
-    </row>
-    <row r="6" spans="2:129" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="127"/>
-      <c r="C6" s="128"/>
-      <c r="D6" s="128"/>
-      <c r="E6" s="128"/>
-      <c r="F6" s="128"/>
-      <c r="G6" s="129"/>
-      <c r="H6" s="136"/>
-      <c r="I6" s="137"/>
-      <c r="J6" s="137"/>
-      <c r="K6" s="138"/>
-      <c r="L6" s="127"/>
-      <c r="M6" s="128"/>
-      <c r="N6" s="129"/>
-      <c r="O6" s="136"/>
-      <c r="P6" s="137"/>
-      <c r="Q6" s="137"/>
-      <c r="R6" s="137"/>
-      <c r="S6" s="137"/>
-      <c r="T6" s="137"/>
-      <c r="U6" s="138"/>
+      <c r="DY5" s="77"/>
+      <c r="DZ5" s="78"/>
+    </row>
+    <row r="6" spans="2:130" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="125"/>
+      <c r="C6" s="126"/>
+      <c r="D6" s="126"/>
+      <c r="E6" s="126"/>
+      <c r="F6" s="126"/>
+      <c r="G6" s="126"/>
+      <c r="H6" s="127"/>
+      <c r="I6" s="134"/>
+      <c r="J6" s="135"/>
+      <c r="K6" s="135"/>
+      <c r="L6" s="136"/>
+      <c r="M6" s="125"/>
+      <c r="N6" s="126"/>
+      <c r="O6" s="127"/>
+      <c r="P6" s="134"/>
+      <c r="Q6" s="135"/>
+      <c r="R6" s="135"/>
+      <c r="S6" s="135"/>
+      <c r="T6" s="135"/>
+      <c r="U6" s="135"/>
       <c r="V6" s="136"/>
-      <c r="W6" s="137"/>
-      <c r="X6" s="137"/>
-      <c r="Y6" s="137"/>
-      <c r="Z6" s="137"/>
-      <c r="AA6" s="137"/>
-      <c r="AB6" s="138"/>
-      <c r="AC6" s="100" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD6" s="76"/>
-      <c r="AE6" s="77"/>
+      <c r="W6" s="134"/>
+      <c r="X6" s="135"/>
+      <c r="Y6" s="135"/>
+      <c r="Z6" s="135"/>
+      <c r="AA6" s="135"/>
+      <c r="AB6" s="135"/>
+      <c r="AC6" s="136"/>
+      <c r="AD6" s="100" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE6" s="76"/>
       <c r="AF6" s="77"/>
       <c r="AG6" s="77"/>
       <c r="AH6" s="77"/>
@@ -2719,95 +2720,98 @@
       <c r="DV6" s="77"/>
       <c r="DW6" s="77"/>
       <c r="DX6" s="77"/>
-      <c r="DY6" s="78"/>
-    </row>
-    <row r="7" spans="2:129" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="101" t="s">
+      <c r="DY6" s="77"/>
+      <c r="DZ6" s="78"/>
+    </row>
+    <row r="7" spans="2:130" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="61" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="102" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="45" t="s">
+      <c r="F7" s="101" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="60" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="103" t="s">
+      <c r="I7" s="59" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="M7" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="N7" s="89" t="s">
+        <v>20</v>
+      </c>
+      <c r="O7" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="P7" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q7" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="R7" s="60" t="s">
+        <v>22</v>
+      </c>
+      <c r="S7" s="60" t="s">
+        <v>23</v>
+      </c>
+      <c r="T7" s="60" t="s">
+        <v>24</v>
+      </c>
+      <c r="U7" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="60" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="104" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="59" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="61" t="s">
+      <c r="V7" s="63" t="s">
+        <v>25</v>
+      </c>
+      <c r="W7" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="62" t="s">
+      <c r="X7" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y7" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="M7" s="89" t="s">
-        <v>21</v>
-      </c>
-      <c r="N7" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="O7" s="59" t="s">
-        <v>37</v>
-      </c>
-      <c r="P7" s="60" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q7" s="60" t="s">
+      <c r="Z7" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="R7" s="60" t="s">
+      <c r="AA7" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="S7" s="60" t="s">
+      <c r="AB7" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC7" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="60" t="s">
-        <v>40</v>
-      </c>
-      <c r="U7" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="V7" s="61" t="s">
-        <v>37</v>
-      </c>
-      <c r="W7" s="60" t="s">
-        <v>38</v>
-      </c>
-      <c r="X7" s="60" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y7" s="60" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z7" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA7" s="60" t="s">
-        <v>40</v>
-      </c>
-      <c r="AB7" s="64" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC7" s="88" t="s">
-        <v>30</v>
-      </c>
-      <c r="AD7" s="79"/>
-      <c r="AE7" s="80"/>
+      <c r="AD7" s="88" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE7" s="79"/>
       <c r="AF7" s="80"/>
       <c r="AG7" s="80"/>
       <c r="AH7" s="80"/>
@@ -2905,39 +2909,40 @@
       <c r="DV7" s="80"/>
       <c r="DW7" s="80"/>
       <c r="DX7" s="80"/>
-      <c r="DY7" s="81"/>
-    </row>
-    <row r="8" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="DY7" s="80"/>
+      <c r="DZ7" s="81"/>
+    </row>
+    <row r="8" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B8" s="14"/>
       <c r="C8" s="90"/>
       <c r="D8" s="90"/>
-      <c r="E8" s="94"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="39"/>
-      <c r="N8" s="41"/>
-      <c r="O8" s="37"/>
-      <c r="P8" s="39"/>
-      <c r="Q8" s="56"/>
+      <c r="E8" s="90"/>
+      <c r="F8" s="94"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="41"/>
+      <c r="P8" s="37"/>
+      <c r="Q8" s="39"/>
       <c r="R8" s="56"/>
       <c r="S8" s="56"/>
-      <c r="T8" s="39"/>
-      <c r="U8" s="53"/>
-      <c r="V8" s="43"/>
-      <c r="W8" s="39"/>
-      <c r="X8" s="56"/>
+      <c r="T8" s="56"/>
+      <c r="U8" s="39"/>
+      <c r="V8" s="53"/>
+      <c r="W8" s="43"/>
+      <c r="X8" s="39"/>
       <c r="Y8" s="56"/>
       <c r="Z8" s="56"/>
-      <c r="AA8" s="39"/>
-      <c r="AB8" s="65"/>
-      <c r="AC8" s="71"/>
-      <c r="AD8" s="82"/>
-      <c r="AE8" s="83"/>
+      <c r="AA8" s="56"/>
+      <c r="AB8" s="39"/>
+      <c r="AC8" s="65"/>
+      <c r="AD8" s="71"/>
+      <c r="AE8" s="82"/>
       <c r="AF8" s="83"/>
       <c r="AG8" s="83"/>
       <c r="AH8" s="83"/>
@@ -3035,1464 +3040,1514 @@
       <c r="DV8" s="83"/>
       <c r="DW8" s="83"/>
       <c r="DX8" s="83"/>
-      <c r="DY8" s="84"/>
-    </row>
-    <row r="9" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="DY8" s="83"/>
+      <c r="DZ8" s="84"/>
+    </row>
+    <row r="9" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B9" s="6"/>
       <c r="C9" s="91"/>
       <c r="D9" s="91"/>
-      <c r="E9" s="95"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="40"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="44"/>
-      <c r="M9" s="40"/>
-      <c r="N9" s="42"/>
-      <c r="O9" s="38"/>
-      <c r="P9" s="40"/>
-      <c r="Q9" s="57"/>
+      <c r="E9" s="91"/>
+      <c r="F9" s="95"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="42"/>
+      <c r="M9" s="44"/>
+      <c r="N9" s="40"/>
+      <c r="O9" s="42"/>
+      <c r="P9" s="38"/>
+      <c r="Q9" s="40"/>
       <c r="R9" s="57"/>
       <c r="S9" s="57"/>
-      <c r="T9" s="40"/>
-      <c r="U9" s="54"/>
-      <c r="V9" s="44"/>
-      <c r="W9" s="40"/>
-      <c r="X9" s="57"/>
+      <c r="T9" s="57"/>
+      <c r="U9" s="40"/>
+      <c r="V9" s="54"/>
+      <c r="W9" s="44"/>
+      <c r="X9" s="40"/>
       <c r="Y9" s="57"/>
       <c r="Z9" s="57"/>
-      <c r="AA9" s="40"/>
-      <c r="AB9" s="66"/>
-    </row>
-    <row r="10" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA9" s="57"/>
+      <c r="AB9" s="40"/>
+      <c r="AC9" s="66"/>
+    </row>
+    <row r="10" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B10" s="6"/>
       <c r="C10" s="91"/>
       <c r="D10" s="91"/>
-      <c r="E10" s="95"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="42"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="42"/>
-      <c r="O10" s="38"/>
-      <c r="P10" s="40"/>
-      <c r="Q10" s="57"/>
+      <c r="E10" s="91"/>
+      <c r="F10" s="95"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="40"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="40"/>
+      <c r="O10" s="42"/>
+      <c r="P10" s="38"/>
+      <c r="Q10" s="40"/>
       <c r="R10" s="57"/>
       <c r="S10" s="57"/>
-      <c r="T10" s="40"/>
-      <c r="U10" s="54"/>
-      <c r="V10" s="44"/>
-      <c r="W10" s="40"/>
-      <c r="X10" s="57"/>
+      <c r="T10" s="57"/>
+      <c r="U10" s="40"/>
+      <c r="V10" s="54"/>
+      <c r="W10" s="44"/>
+      <c r="X10" s="40"/>
       <c r="Y10" s="57"/>
       <c r="Z10" s="57"/>
-      <c r="AA10" s="40"/>
-      <c r="AB10" s="66"/>
-    </row>
-    <row r="11" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA10" s="57"/>
+      <c r="AB10" s="40"/>
+      <c r="AC10" s="66"/>
+    </row>
+    <row r="11" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B11" s="6"/>
       <c r="C11" s="91"/>
       <c r="D11" s="91"/>
-      <c r="E11" s="95"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="38"/>
-      <c r="I11" s="44"/>
-      <c r="J11" s="40"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="44"/>
-      <c r="M11" s="40"/>
-      <c r="N11" s="42"/>
-      <c r="O11" s="38"/>
-      <c r="P11" s="40"/>
-      <c r="Q11" s="57"/>
+      <c r="E11" s="91"/>
+      <c r="F11" s="95"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="42"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="40"/>
+      <c r="O11" s="42"/>
+      <c r="P11" s="38"/>
+      <c r="Q11" s="40"/>
       <c r="R11" s="57"/>
       <c r="S11" s="57"/>
-      <c r="T11" s="40"/>
-      <c r="U11" s="54"/>
-      <c r="V11" s="44"/>
-      <c r="W11" s="40"/>
-      <c r="X11" s="57"/>
+      <c r="T11" s="57"/>
+      <c r="U11" s="40"/>
+      <c r="V11" s="54"/>
+      <c r="W11" s="44"/>
+      <c r="X11" s="40"/>
       <c r="Y11" s="57"/>
       <c r="Z11" s="57"/>
-      <c r="AA11" s="40"/>
-      <c r="AB11" s="66"/>
-    </row>
-    <row r="12" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA11" s="57"/>
+      <c r="AB11" s="40"/>
+      <c r="AC11" s="66"/>
+    </row>
+    <row r="12" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B12" s="6"/>
       <c r="C12" s="91"/>
       <c r="D12" s="91"/>
-      <c r="E12" s="95"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="38"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="44"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="42"/>
-      <c r="O12" s="38"/>
-      <c r="P12" s="40"/>
-      <c r="Q12" s="57"/>
+      <c r="E12" s="91"/>
+      <c r="F12" s="95"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="42"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="40"/>
+      <c r="O12" s="42"/>
+      <c r="P12" s="38"/>
+      <c r="Q12" s="40"/>
       <c r="R12" s="57"/>
       <c r="S12" s="57"/>
-      <c r="T12" s="40"/>
-      <c r="U12" s="54"/>
-      <c r="V12" s="44"/>
-      <c r="W12" s="40"/>
-      <c r="X12" s="57"/>
+      <c r="T12" s="57"/>
+      <c r="U12" s="40"/>
+      <c r="V12" s="54"/>
+      <c r="W12" s="44"/>
+      <c r="X12" s="40"/>
       <c r="Y12" s="57"/>
       <c r="Z12" s="57"/>
-      <c r="AA12" s="40"/>
-      <c r="AB12" s="66"/>
-    </row>
-    <row r="13" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA12" s="57"/>
+      <c r="AB12" s="40"/>
+      <c r="AC12" s="66"/>
+    </row>
+    <row r="13" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B13" s="6"/>
       <c r="C13" s="91"/>
       <c r="D13" s="91"/>
-      <c r="E13" s="95"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="44"/>
-      <c r="J13" s="40"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="44"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="42"/>
-      <c r="O13" s="38"/>
-      <c r="P13" s="40"/>
-      <c r="Q13" s="57"/>
+      <c r="E13" s="91"/>
+      <c r="F13" s="95"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="40"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="40"/>
+      <c r="O13" s="42"/>
+      <c r="P13" s="38"/>
+      <c r="Q13" s="40"/>
       <c r="R13" s="57"/>
       <c r="S13" s="57"/>
-      <c r="T13" s="40"/>
-      <c r="U13" s="54"/>
-      <c r="V13" s="44"/>
-      <c r="W13" s="40"/>
-      <c r="X13" s="57"/>
+      <c r="T13" s="57"/>
+      <c r="U13" s="40"/>
+      <c r="V13" s="54"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="40"/>
       <c r="Y13" s="57"/>
       <c r="Z13" s="57"/>
-      <c r="AA13" s="40"/>
-      <c r="AB13" s="66"/>
-    </row>
-    <row r="14" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA13" s="57"/>
+      <c r="AB13" s="40"/>
+      <c r="AC13" s="66"/>
+    </row>
+    <row r="14" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B14" s="6"/>
       <c r="C14" s="91"/>
       <c r="D14" s="91"/>
-      <c r="E14" s="95"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="40"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="44"/>
-      <c r="M14" s="40"/>
-      <c r="N14" s="42"/>
-      <c r="O14" s="38"/>
-      <c r="P14" s="40"/>
-      <c r="Q14" s="57"/>
+      <c r="E14" s="91"/>
+      <c r="F14" s="95"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="44"/>
+      <c r="N14" s="40"/>
+      <c r="O14" s="42"/>
+      <c r="P14" s="38"/>
+      <c r="Q14" s="40"/>
       <c r="R14" s="57"/>
       <c r="S14" s="57"/>
-      <c r="T14" s="40"/>
-      <c r="U14" s="54"/>
-      <c r="V14" s="44"/>
-      <c r="W14" s="40"/>
-      <c r="X14" s="57"/>
+      <c r="T14" s="57"/>
+      <c r="U14" s="40"/>
+      <c r="V14" s="54"/>
+      <c r="W14" s="44"/>
+      <c r="X14" s="40"/>
       <c r="Y14" s="57"/>
       <c r="Z14" s="57"/>
-      <c r="AA14" s="40"/>
-      <c r="AB14" s="66"/>
-    </row>
-    <row r="15" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA14" s="57"/>
+      <c r="AB14" s="40"/>
+      <c r="AC14" s="66"/>
+    </row>
+    <row r="15" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B15" s="6"/>
       <c r="C15" s="91"/>
       <c r="D15" s="91"/>
-      <c r="E15" s="95"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="44"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="44"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="42"/>
-      <c r="O15" s="38"/>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="57"/>
+      <c r="E15" s="91"/>
+      <c r="F15" s="95"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="40"/>
+      <c r="L15" s="42"/>
+      <c r="M15" s="44"/>
+      <c r="N15" s="40"/>
+      <c r="O15" s="42"/>
+      <c r="P15" s="38"/>
+      <c r="Q15" s="40"/>
       <c r="R15" s="57"/>
       <c r="S15" s="57"/>
-      <c r="T15" s="40"/>
-      <c r="U15" s="54"/>
-      <c r="V15" s="44"/>
-      <c r="W15" s="40"/>
-      <c r="X15" s="57"/>
+      <c r="T15" s="57"/>
+      <c r="U15" s="40"/>
+      <c r="V15" s="54"/>
+      <c r="W15" s="44"/>
+      <c r="X15" s="40"/>
       <c r="Y15" s="57"/>
       <c r="Z15" s="57"/>
-      <c r="AA15" s="40"/>
-      <c r="AB15" s="66"/>
-    </row>
-    <row r="16" spans="2:129" x14ac:dyDescent="0.25">
+      <c r="AA15" s="57"/>
+      <c r="AB15" s="40"/>
+      <c r="AC15" s="66"/>
+    </row>
+    <row r="16" spans="2:130" x14ac:dyDescent="0.3">
       <c r="B16" s="6"/>
       <c r="C16" s="91"/>
       <c r="D16" s="91"/>
-      <c r="E16" s="95"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="44"/>
-      <c r="J16" s="40"/>
-      <c r="K16" s="42"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="40"/>
-      <c r="N16" s="42"/>
-      <c r="O16" s="38"/>
-      <c r="P16" s="40"/>
-      <c r="Q16" s="57"/>
+      <c r="E16" s="91"/>
+      <c r="F16" s="95"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="44"/>
+      <c r="K16" s="40"/>
+      <c r="L16" s="42"/>
+      <c r="M16" s="44"/>
+      <c r="N16" s="40"/>
+      <c r="O16" s="42"/>
+      <c r="P16" s="38"/>
+      <c r="Q16" s="40"/>
       <c r="R16" s="57"/>
       <c r="S16" s="57"/>
-      <c r="T16" s="40"/>
-      <c r="U16" s="54"/>
-      <c r="V16" s="44"/>
-      <c r="W16" s="40"/>
-      <c r="X16" s="57"/>
+      <c r="T16" s="57"/>
+      <c r="U16" s="40"/>
+      <c r="V16" s="54"/>
+      <c r="W16" s="44"/>
+      <c r="X16" s="40"/>
       <c r="Y16" s="57"/>
       <c r="Z16" s="57"/>
-      <c r="AA16" s="40"/>
-      <c r="AB16" s="66"/>
-    </row>
-    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA16" s="57"/>
+      <c r="AB16" s="40"/>
+      <c r="AC16" s="66"/>
+    </row>
+    <row r="17" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B17" s="6"/>
       <c r="C17" s="91"/>
       <c r="D17" s="91"/>
-      <c r="E17" s="95"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="44"/>
-      <c r="J17" s="40"/>
-      <c r="K17" s="42"/>
-      <c r="L17" s="44"/>
-      <c r="M17" s="40"/>
-      <c r="N17" s="42"/>
-      <c r="O17" s="38"/>
-      <c r="P17" s="40"/>
-      <c r="Q17" s="57"/>
+      <c r="E17" s="91"/>
+      <c r="F17" s="95"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="40"/>
+      <c r="L17" s="42"/>
+      <c r="M17" s="44"/>
+      <c r="N17" s="40"/>
+      <c r="O17" s="42"/>
+      <c r="P17" s="38"/>
+      <c r="Q17" s="40"/>
       <c r="R17" s="57"/>
       <c r="S17" s="57"/>
-      <c r="T17" s="40"/>
-      <c r="U17" s="54"/>
-      <c r="V17" s="44"/>
-      <c r="W17" s="40"/>
-      <c r="X17" s="57"/>
+      <c r="T17" s="57"/>
+      <c r="U17" s="40"/>
+      <c r="V17" s="54"/>
+      <c r="W17" s="44"/>
+      <c r="X17" s="40"/>
       <c r="Y17" s="57"/>
       <c r="Z17" s="57"/>
-      <c r="AA17" s="40"/>
-      <c r="AB17" s="66"/>
-    </row>
-    <row r="18" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA17" s="57"/>
+      <c r="AB17" s="40"/>
+      <c r="AC17" s="66"/>
+    </row>
+    <row r="18" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B18" s="6"/>
       <c r="C18" s="91"/>
       <c r="D18" s="91"/>
-      <c r="E18" s="95"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="40"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="44"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="42"/>
-      <c r="O18" s="38"/>
-      <c r="P18" s="40"/>
-      <c r="Q18" s="57"/>
+      <c r="E18" s="91"/>
+      <c r="F18" s="95"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="42"/>
+      <c r="M18" s="44"/>
+      <c r="N18" s="40"/>
+      <c r="O18" s="42"/>
+      <c r="P18" s="38"/>
+      <c r="Q18" s="40"/>
       <c r="R18" s="57"/>
       <c r="S18" s="57"/>
-      <c r="T18" s="40"/>
-      <c r="U18" s="54"/>
-      <c r="V18" s="44"/>
-      <c r="W18" s="40"/>
-      <c r="X18" s="57"/>
+      <c r="T18" s="57"/>
+      <c r="U18" s="40"/>
+      <c r="V18" s="54"/>
+      <c r="W18" s="44"/>
+      <c r="X18" s="40"/>
       <c r="Y18" s="57"/>
       <c r="Z18" s="57"/>
-      <c r="AA18" s="40"/>
-      <c r="AB18" s="66"/>
-    </row>
-    <row r="19" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA18" s="57"/>
+      <c r="AB18" s="40"/>
+      <c r="AC18" s="66"/>
+    </row>
+    <row r="19" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B19" s="6"/>
       <c r="C19" s="91"/>
       <c r="D19" s="91"/>
-      <c r="E19" s="95"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="42"/>
-      <c r="L19" s="44"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="42"/>
-      <c r="O19" s="38"/>
-      <c r="P19" s="40"/>
-      <c r="Q19" s="57"/>
+      <c r="E19" s="91"/>
+      <c r="F19" s="95"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="38"/>
+      <c r="J19" s="44"/>
+      <c r="K19" s="40"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="44"/>
+      <c r="N19" s="40"/>
+      <c r="O19" s="42"/>
+      <c r="P19" s="38"/>
+      <c r="Q19" s="40"/>
       <c r="R19" s="57"/>
       <c r="S19" s="57"/>
-      <c r="T19" s="40"/>
-      <c r="U19" s="54"/>
-      <c r="V19" s="44"/>
-      <c r="W19" s="40"/>
-      <c r="X19" s="57"/>
+      <c r="T19" s="57"/>
+      <c r="U19" s="40"/>
+      <c r="V19" s="54"/>
+      <c r="W19" s="44"/>
+      <c r="X19" s="40"/>
       <c r="Y19" s="57"/>
       <c r="Z19" s="57"/>
-      <c r="AA19" s="40"/>
-      <c r="AB19" s="66"/>
-    </row>
-    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA19" s="57"/>
+      <c r="AB19" s="40"/>
+      <c r="AC19" s="66"/>
+    </row>
+    <row r="20" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B20" s="6"/>
       <c r="C20" s="91"/>
       <c r="D20" s="91"/>
-      <c r="E20" s="95"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="44"/>
-      <c r="J20" s="40"/>
-      <c r="K20" s="42"/>
-      <c r="L20" s="44"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="38"/>
-      <c r="P20" s="40"/>
-      <c r="Q20" s="57"/>
+      <c r="E20" s="91"/>
+      <c r="F20" s="95"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="38"/>
+      <c r="J20" s="44"/>
+      <c r="K20" s="40"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="44"/>
+      <c r="N20" s="40"/>
+      <c r="O20" s="42"/>
+      <c r="P20" s="38"/>
+      <c r="Q20" s="40"/>
       <c r="R20" s="57"/>
       <c r="S20" s="57"/>
-      <c r="T20" s="40"/>
-      <c r="U20" s="54"/>
-      <c r="V20" s="44"/>
-      <c r="W20" s="40"/>
-      <c r="X20" s="57"/>
+      <c r="T20" s="57"/>
+      <c r="U20" s="40"/>
+      <c r="V20" s="54"/>
+      <c r="W20" s="44"/>
+      <c r="X20" s="40"/>
       <c r="Y20" s="57"/>
       <c r="Z20" s="57"/>
-      <c r="AA20" s="40"/>
-      <c r="AB20" s="66"/>
-    </row>
-    <row r="21" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA20" s="57"/>
+      <c r="AB20" s="40"/>
+      <c r="AC20" s="66"/>
+    </row>
+    <row r="21" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B21" s="6"/>
       <c r="C21" s="91"/>
       <c r="D21" s="91"/>
-      <c r="E21" s="95"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="40"/>
-      <c r="K21" s="42"/>
-      <c r="L21" s="44"/>
-      <c r="M21" s="40"/>
-      <c r="N21" s="42"/>
-      <c r="O21" s="38"/>
-      <c r="P21" s="40"/>
-      <c r="Q21" s="57"/>
+      <c r="E21" s="91"/>
+      <c r="F21" s="95"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="38"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="42"/>
+      <c r="M21" s="44"/>
+      <c r="N21" s="40"/>
+      <c r="O21" s="42"/>
+      <c r="P21" s="38"/>
+      <c r="Q21" s="40"/>
       <c r="R21" s="57"/>
       <c r="S21" s="57"/>
-      <c r="T21" s="40"/>
-      <c r="U21" s="54"/>
-      <c r="V21" s="44"/>
-      <c r="W21" s="40"/>
-      <c r="X21" s="57"/>
+      <c r="T21" s="57"/>
+      <c r="U21" s="40"/>
+      <c r="V21" s="54"/>
+      <c r="W21" s="44"/>
+      <c r="X21" s="40"/>
       <c r="Y21" s="57"/>
       <c r="Z21" s="57"/>
-      <c r="AA21" s="40"/>
-      <c r="AB21" s="66"/>
-    </row>
-    <row r="22" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA21" s="57"/>
+      <c r="AB21" s="40"/>
+      <c r="AC21" s="66"/>
+    </row>
+    <row r="22" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B22" s="6"/>
       <c r="C22" s="91"/>
       <c r="D22" s="91"/>
-      <c r="E22" s="95"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="44"/>
-      <c r="J22" s="40"/>
-      <c r="K22" s="42"/>
-      <c r="L22" s="44"/>
-      <c r="M22" s="40"/>
-      <c r="N22" s="42"/>
-      <c r="O22" s="38"/>
-      <c r="P22" s="40"/>
-      <c r="Q22" s="57"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="95"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="38"/>
+      <c r="J22" s="44"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="42"/>
+      <c r="M22" s="44"/>
+      <c r="N22" s="40"/>
+      <c r="O22" s="42"/>
+      <c r="P22" s="38"/>
+      <c r="Q22" s="40"/>
       <c r="R22" s="57"/>
       <c r="S22" s="57"/>
-      <c r="T22" s="40"/>
-      <c r="U22" s="54"/>
-      <c r="V22" s="44"/>
-      <c r="W22" s="40"/>
-      <c r="X22" s="57"/>
+      <c r="T22" s="57"/>
+      <c r="U22" s="40"/>
+      <c r="V22" s="54"/>
+      <c r="W22" s="44"/>
+      <c r="X22" s="40"/>
       <c r="Y22" s="57"/>
       <c r="Z22" s="57"/>
-      <c r="AA22" s="40"/>
-      <c r="AB22" s="66"/>
-    </row>
-    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA22" s="57"/>
+      <c r="AB22" s="40"/>
+      <c r="AC22" s="66"/>
+    </row>
+    <row r="23" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B23" s="6"/>
       <c r="C23" s="91"/>
       <c r="D23" s="91"/>
-      <c r="E23" s="95"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="40"/>
-      <c r="K23" s="42"/>
-      <c r="L23" s="44"/>
-      <c r="M23" s="40"/>
-      <c r="N23" s="42"/>
-      <c r="O23" s="38"/>
-      <c r="P23" s="40"/>
-      <c r="Q23" s="57"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="95"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="38"/>
+      <c r="J23" s="44"/>
+      <c r="K23" s="40"/>
+      <c r="L23" s="42"/>
+      <c r="M23" s="44"/>
+      <c r="N23" s="40"/>
+      <c r="O23" s="42"/>
+      <c r="P23" s="38"/>
+      <c r="Q23" s="40"/>
       <c r="R23" s="57"/>
       <c r="S23" s="57"/>
-      <c r="T23" s="40"/>
-      <c r="U23" s="54"/>
-      <c r="V23" s="44"/>
-      <c r="W23" s="40"/>
-      <c r="X23" s="57"/>
+      <c r="T23" s="57"/>
+      <c r="U23" s="40"/>
+      <c r="V23" s="54"/>
+      <c r="W23" s="44"/>
+      <c r="X23" s="40"/>
       <c r="Y23" s="57"/>
       <c r="Z23" s="57"/>
-      <c r="AA23" s="40"/>
-      <c r="AB23" s="66"/>
-    </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA23" s="57"/>
+      <c r="AB23" s="40"/>
+      <c r="AC23" s="66"/>
+    </row>
+    <row r="24" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B24" s="6"/>
       <c r="C24" s="91"/>
       <c r="D24" s="91"/>
-      <c r="E24" s="95"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="40"/>
-      <c r="K24" s="42"/>
-      <c r="L24" s="44"/>
-      <c r="M24" s="40"/>
-      <c r="N24" s="42"/>
-      <c r="O24" s="38"/>
-      <c r="P24" s="40"/>
-      <c r="Q24" s="57"/>
+      <c r="E24" s="91"/>
+      <c r="F24" s="95"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="38"/>
+      <c r="J24" s="44"/>
+      <c r="K24" s="40"/>
+      <c r="L24" s="42"/>
+      <c r="M24" s="44"/>
+      <c r="N24" s="40"/>
+      <c r="O24" s="42"/>
+      <c r="P24" s="38"/>
+      <c r="Q24" s="40"/>
       <c r="R24" s="57"/>
       <c r="S24" s="57"/>
-      <c r="T24" s="40"/>
-      <c r="U24" s="54"/>
-      <c r="V24" s="44"/>
-      <c r="W24" s="40"/>
-      <c r="X24" s="57"/>
+      <c r="T24" s="57"/>
+      <c r="U24" s="40"/>
+      <c r="V24" s="54"/>
+      <c r="W24" s="44"/>
+      <c r="X24" s="40"/>
       <c r="Y24" s="57"/>
       <c r="Z24" s="57"/>
-      <c r="AA24" s="40"/>
-      <c r="AB24" s="66"/>
-    </row>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA24" s="57"/>
+      <c r="AB24" s="40"/>
+      <c r="AC24" s="66"/>
+    </row>
+    <row r="25" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B25" s="6"/>
       <c r="C25" s="91"/>
       <c r="D25" s="91"/>
-      <c r="E25" s="95"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="44"/>
-      <c r="J25" s="40"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="44"/>
-      <c r="M25" s="40"/>
-      <c r="N25" s="42"/>
-      <c r="O25" s="38"/>
-      <c r="P25" s="40"/>
-      <c r="Q25" s="57"/>
+      <c r="E25" s="91"/>
+      <c r="F25" s="95"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="40"/>
+      <c r="L25" s="42"/>
+      <c r="M25" s="44"/>
+      <c r="N25" s="40"/>
+      <c r="O25" s="42"/>
+      <c r="P25" s="38"/>
+      <c r="Q25" s="40"/>
       <c r="R25" s="57"/>
       <c r="S25" s="57"/>
-      <c r="T25" s="40"/>
-      <c r="U25" s="54"/>
-      <c r="V25" s="44"/>
-      <c r="W25" s="40"/>
-      <c r="X25" s="57"/>
+      <c r="T25" s="57"/>
+      <c r="U25" s="40"/>
+      <c r="V25" s="54"/>
+      <c r="W25" s="44"/>
+      <c r="X25" s="40"/>
       <c r="Y25" s="57"/>
       <c r="Z25" s="57"/>
-      <c r="AA25" s="40"/>
-      <c r="AB25" s="66"/>
-    </row>
-    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA25" s="57"/>
+      <c r="AB25" s="40"/>
+      <c r="AC25" s="66"/>
+    </row>
+    <row r="26" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B26" s="6"/>
       <c r="C26" s="91"/>
       <c r="D26" s="91"/>
-      <c r="E26" s="95"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="38"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="40"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="40"/>
-      <c r="N26" s="42"/>
-      <c r="O26" s="38"/>
-      <c r="P26" s="40"/>
-      <c r="Q26" s="57"/>
+      <c r="E26" s="91"/>
+      <c r="F26" s="95"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="44"/>
+      <c r="N26" s="40"/>
+      <c r="O26" s="42"/>
+      <c r="P26" s="38"/>
+      <c r="Q26" s="40"/>
       <c r="R26" s="57"/>
       <c r="S26" s="57"/>
-      <c r="T26" s="40"/>
-      <c r="U26" s="54"/>
-      <c r="V26" s="44"/>
-      <c r="W26" s="40"/>
-      <c r="X26" s="57"/>
+      <c r="T26" s="57"/>
+      <c r="U26" s="40"/>
+      <c r="V26" s="54"/>
+      <c r="W26" s="44"/>
+      <c r="X26" s="40"/>
       <c r="Y26" s="57"/>
       <c r="Z26" s="57"/>
-      <c r="AA26" s="40"/>
-      <c r="AB26" s="66"/>
-    </row>
-    <row r="27" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA26" s="57"/>
+      <c r="AB26" s="40"/>
+      <c r="AC26" s="66"/>
+    </row>
+    <row r="27" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B27" s="6"/>
       <c r="C27" s="91"/>
       <c r="D27" s="91"/>
-      <c r="E27" s="95"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="44"/>
-      <c r="J27" s="40"/>
-      <c r="K27" s="42"/>
-      <c r="L27" s="44"/>
-      <c r="M27" s="40"/>
-      <c r="N27" s="42"/>
-      <c r="O27" s="38"/>
-      <c r="P27" s="40"/>
-      <c r="Q27" s="57"/>
+      <c r="E27" s="91"/>
+      <c r="F27" s="95"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="42"/>
+      <c r="M27" s="44"/>
+      <c r="N27" s="40"/>
+      <c r="O27" s="42"/>
+      <c r="P27" s="38"/>
+      <c r="Q27" s="40"/>
       <c r="R27" s="57"/>
       <c r="S27" s="57"/>
-      <c r="T27" s="40"/>
-      <c r="U27" s="54"/>
-      <c r="V27" s="44"/>
-      <c r="W27" s="40"/>
-      <c r="X27" s="57"/>
+      <c r="T27" s="57"/>
+      <c r="U27" s="40"/>
+      <c r="V27" s="54"/>
+      <c r="W27" s="44"/>
+      <c r="X27" s="40"/>
       <c r="Y27" s="57"/>
       <c r="Z27" s="57"/>
-      <c r="AA27" s="40"/>
-      <c r="AB27" s="66"/>
-    </row>
-    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA27" s="57"/>
+      <c r="AB27" s="40"/>
+      <c r="AC27" s="66"/>
+    </row>
+    <row r="28" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B28" s="6"/>
       <c r="C28" s="91"/>
       <c r="D28" s="91"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="38"/>
-      <c r="I28" s="44"/>
-      <c r="J28" s="40"/>
-      <c r="K28" s="42"/>
-      <c r="L28" s="44"/>
-      <c r="M28" s="40"/>
-      <c r="N28" s="42"/>
-      <c r="O28" s="38"/>
-      <c r="P28" s="40"/>
-      <c r="Q28" s="57"/>
+      <c r="E28" s="91"/>
+      <c r="F28" s="95"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="40"/>
+      <c r="L28" s="42"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="40"/>
+      <c r="O28" s="42"/>
+      <c r="P28" s="38"/>
+      <c r="Q28" s="40"/>
       <c r="R28" s="57"/>
       <c r="S28" s="57"/>
-      <c r="T28" s="40"/>
-      <c r="U28" s="54"/>
-      <c r="V28" s="44"/>
-      <c r="W28" s="40"/>
-      <c r="X28" s="57"/>
+      <c r="T28" s="57"/>
+      <c r="U28" s="40"/>
+      <c r="V28" s="54"/>
+      <c r="W28" s="44"/>
+      <c r="X28" s="40"/>
       <c r="Y28" s="57"/>
       <c r="Z28" s="57"/>
-      <c r="AA28" s="40"/>
-      <c r="AB28" s="66"/>
-    </row>
-    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA28" s="57"/>
+      <c r="AB28" s="40"/>
+      <c r="AC28" s="66"/>
+    </row>
+    <row r="29" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B29" s="6"/>
       <c r="C29" s="91"/>
       <c r="D29" s="91"/>
-      <c r="E29" s="95"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="38"/>
-      <c r="I29" s="44"/>
-      <c r="J29" s="40"/>
-      <c r="K29" s="42"/>
-      <c r="L29" s="44"/>
-      <c r="M29" s="40"/>
-      <c r="N29" s="42"/>
-      <c r="O29" s="38"/>
-      <c r="P29" s="40"/>
-      <c r="Q29" s="57"/>
+      <c r="E29" s="91"/>
+      <c r="F29" s="95"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="44"/>
+      <c r="K29" s="40"/>
+      <c r="L29" s="42"/>
+      <c r="M29" s="44"/>
+      <c r="N29" s="40"/>
+      <c r="O29" s="42"/>
+      <c r="P29" s="38"/>
+      <c r="Q29" s="40"/>
       <c r="R29" s="57"/>
       <c r="S29" s="57"/>
-      <c r="T29" s="40"/>
-      <c r="U29" s="54"/>
-      <c r="V29" s="44"/>
-      <c r="W29" s="40"/>
-      <c r="X29" s="57"/>
+      <c r="T29" s="57"/>
+      <c r="U29" s="40"/>
+      <c r="V29" s="54"/>
+      <c r="W29" s="44"/>
+      <c r="X29" s="40"/>
       <c r="Y29" s="57"/>
       <c r="Z29" s="57"/>
-      <c r="AA29" s="40"/>
-      <c r="AB29" s="66"/>
-    </row>
-    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA29" s="57"/>
+      <c r="AB29" s="40"/>
+      <c r="AC29" s="66"/>
+    </row>
+    <row r="30" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B30" s="6"/>
       <c r="C30" s="91"/>
       <c r="D30" s="91"/>
-      <c r="E30" s="95"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="38"/>
-      <c r="I30" s="44"/>
-      <c r="J30" s="40"/>
-      <c r="K30" s="42"/>
-      <c r="L30" s="44"/>
-      <c r="M30" s="40"/>
-      <c r="N30" s="42"/>
-      <c r="O30" s="38"/>
-      <c r="P30" s="40"/>
-      <c r="Q30" s="57"/>
+      <c r="E30" s="91"/>
+      <c r="F30" s="95"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="38"/>
+      <c r="J30" s="44"/>
+      <c r="K30" s="40"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="44"/>
+      <c r="N30" s="40"/>
+      <c r="O30" s="42"/>
+      <c r="P30" s="38"/>
+      <c r="Q30" s="40"/>
       <c r="R30" s="57"/>
       <c r="S30" s="57"/>
-      <c r="T30" s="40"/>
-      <c r="U30" s="54"/>
-      <c r="V30" s="44"/>
-      <c r="W30" s="40"/>
-      <c r="X30" s="57"/>
+      <c r="T30" s="57"/>
+      <c r="U30" s="40"/>
+      <c r="V30" s="54"/>
+      <c r="W30" s="44"/>
+      <c r="X30" s="40"/>
       <c r="Y30" s="57"/>
       <c r="Z30" s="57"/>
-      <c r="AA30" s="40"/>
-      <c r="AB30" s="66"/>
-    </row>
-    <row r="31" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA30" s="57"/>
+      <c r="AB30" s="40"/>
+      <c r="AC30" s="66"/>
+    </row>
+    <row r="31" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B31" s="6"/>
       <c r="C31" s="91"/>
       <c r="D31" s="91"/>
-      <c r="E31" s="95"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="38"/>
-      <c r="I31" s="44"/>
-      <c r="J31" s="40"/>
-      <c r="K31" s="42"/>
-      <c r="L31" s="44"/>
-      <c r="M31" s="40"/>
-      <c r="N31" s="42"/>
-      <c r="O31" s="38"/>
-      <c r="P31" s="40"/>
-      <c r="Q31" s="57"/>
+      <c r="E31" s="91"/>
+      <c r="F31" s="95"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="38"/>
+      <c r="J31" s="44"/>
+      <c r="K31" s="40"/>
+      <c r="L31" s="42"/>
+      <c r="M31" s="44"/>
+      <c r="N31" s="40"/>
+      <c r="O31" s="42"/>
+      <c r="P31" s="38"/>
+      <c r="Q31" s="40"/>
       <c r="R31" s="57"/>
       <c r="S31" s="57"/>
-      <c r="T31" s="40"/>
-      <c r="U31" s="54"/>
-      <c r="V31" s="44"/>
-      <c r="W31" s="40"/>
-      <c r="X31" s="57"/>
+      <c r="T31" s="57"/>
+      <c r="U31" s="40"/>
+      <c r="V31" s="54"/>
+      <c r="W31" s="44"/>
+      <c r="X31" s="40"/>
       <c r="Y31" s="57"/>
       <c r="Z31" s="57"/>
-      <c r="AA31" s="40"/>
-      <c r="AB31" s="66"/>
-    </row>
-    <row r="32" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA31" s="57"/>
+      <c r="AB31" s="40"/>
+      <c r="AC31" s="66"/>
+    </row>
+    <row r="32" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B32" s="6"/>
       <c r="C32" s="91"/>
       <c r="D32" s="91"/>
-      <c r="E32" s="95"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="9"/>
-      <c r="H32" s="38"/>
-      <c r="I32" s="44"/>
-      <c r="J32" s="40"/>
-      <c r="K32" s="42"/>
-      <c r="L32" s="44"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="42"/>
-      <c r="O32" s="38"/>
-      <c r="P32" s="40"/>
-      <c r="Q32" s="57"/>
+      <c r="E32" s="91"/>
+      <c r="F32" s="95"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="38"/>
+      <c r="J32" s="44"/>
+      <c r="K32" s="40"/>
+      <c r="L32" s="42"/>
+      <c r="M32" s="44"/>
+      <c r="N32" s="40"/>
+      <c r="O32" s="42"/>
+      <c r="P32" s="38"/>
+      <c r="Q32" s="40"/>
       <c r="R32" s="57"/>
       <c r="S32" s="57"/>
-      <c r="T32" s="40"/>
-      <c r="U32" s="54"/>
-      <c r="V32" s="44"/>
-      <c r="W32" s="40"/>
-      <c r="X32" s="57"/>
+      <c r="T32" s="57"/>
+      <c r="U32" s="40"/>
+      <c r="V32" s="54"/>
+      <c r="W32" s="44"/>
+      <c r="X32" s="40"/>
       <c r="Y32" s="57"/>
       <c r="Z32" s="57"/>
-      <c r="AA32" s="40"/>
-      <c r="AB32" s="66"/>
-    </row>
-    <row r="33" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA32" s="57"/>
+      <c r="AB32" s="40"/>
+      <c r="AC32" s="66"/>
+    </row>
+    <row r="33" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B33" s="6"/>
       <c r="C33" s="91"/>
       <c r="D33" s="91"/>
-      <c r="E33" s="95"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="9"/>
-      <c r="H33" s="38"/>
-      <c r="I33" s="44"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="42"/>
-      <c r="L33" s="44"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="42"/>
-      <c r="O33" s="38"/>
-      <c r="P33" s="40"/>
-      <c r="Q33" s="57"/>
+      <c r="E33" s="91"/>
+      <c r="F33" s="95"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="38"/>
+      <c r="J33" s="44"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="44"/>
+      <c r="N33" s="40"/>
+      <c r="O33" s="42"/>
+      <c r="P33" s="38"/>
+      <c r="Q33" s="40"/>
       <c r="R33" s="57"/>
       <c r="S33" s="57"/>
-      <c r="T33" s="40"/>
-      <c r="U33" s="54"/>
-      <c r="V33" s="44"/>
-      <c r="W33" s="40"/>
-      <c r="X33" s="57"/>
+      <c r="T33" s="57"/>
+      <c r="U33" s="40"/>
+      <c r="V33" s="54"/>
+      <c r="W33" s="44"/>
+      <c r="X33" s="40"/>
       <c r="Y33" s="57"/>
       <c r="Z33" s="57"/>
-      <c r="AA33" s="40"/>
-      <c r="AB33" s="66"/>
-    </row>
-    <row r="34" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA33" s="57"/>
+      <c r="AB33" s="40"/>
+      <c r="AC33" s="66"/>
+    </row>
+    <row r="34" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B34" s="6"/>
       <c r="C34" s="91"/>
       <c r="D34" s="91"/>
-      <c r="E34" s="95"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="38"/>
-      <c r="I34" s="44"/>
-      <c r="J34" s="40"/>
-      <c r="K34" s="42"/>
-      <c r="L34" s="44"/>
-      <c r="M34" s="40"/>
-      <c r="N34" s="42"/>
-      <c r="O34" s="38"/>
-      <c r="P34" s="40"/>
-      <c r="Q34" s="57"/>
+      <c r="E34" s="91"/>
+      <c r="F34" s="95"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="38"/>
+      <c r="J34" s="44"/>
+      <c r="K34" s="40"/>
+      <c r="L34" s="42"/>
+      <c r="M34" s="44"/>
+      <c r="N34" s="40"/>
+      <c r="O34" s="42"/>
+      <c r="P34" s="38"/>
+      <c r="Q34" s="40"/>
       <c r="R34" s="57"/>
       <c r="S34" s="57"/>
-      <c r="T34" s="40"/>
-      <c r="U34" s="54"/>
-      <c r="V34" s="44"/>
-      <c r="W34" s="40"/>
-      <c r="X34" s="57"/>
+      <c r="T34" s="57"/>
+      <c r="U34" s="40"/>
+      <c r="V34" s="54"/>
+      <c r="W34" s="44"/>
+      <c r="X34" s="40"/>
       <c r="Y34" s="57"/>
       <c r="Z34" s="57"/>
-      <c r="AA34" s="40"/>
-      <c r="AB34" s="66"/>
-    </row>
-    <row r="35" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA34" s="57"/>
+      <c r="AB34" s="40"/>
+      <c r="AC34" s="66"/>
+    </row>
+    <row r="35" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B35" s="6"/>
       <c r="C35" s="91"/>
       <c r="D35" s="91"/>
-      <c r="E35" s="95"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="38"/>
-      <c r="I35" s="44"/>
-      <c r="J35" s="40"/>
-      <c r="K35" s="42"/>
-      <c r="L35" s="44"/>
-      <c r="M35" s="40"/>
-      <c r="N35" s="42"/>
-      <c r="O35" s="38"/>
-      <c r="P35" s="40"/>
-      <c r="Q35" s="57"/>
+      <c r="E35" s="91"/>
+      <c r="F35" s="95"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="38"/>
+      <c r="J35" s="44"/>
+      <c r="K35" s="40"/>
+      <c r="L35" s="42"/>
+      <c r="M35" s="44"/>
+      <c r="N35" s="40"/>
+      <c r="O35" s="42"/>
+      <c r="P35" s="38"/>
+      <c r="Q35" s="40"/>
       <c r="R35" s="57"/>
       <c r="S35" s="57"/>
-      <c r="T35" s="40"/>
-      <c r="U35" s="54"/>
-      <c r="V35" s="44"/>
-      <c r="W35" s="40"/>
-      <c r="X35" s="57"/>
+      <c r="T35" s="57"/>
+      <c r="U35" s="40"/>
+      <c r="V35" s="54"/>
+      <c r="W35" s="44"/>
+      <c r="X35" s="40"/>
       <c r="Y35" s="57"/>
       <c r="Z35" s="57"/>
-      <c r="AA35" s="40"/>
-      <c r="AB35" s="66"/>
-    </row>
-    <row r="36" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA35" s="57"/>
+      <c r="AB35" s="40"/>
+      <c r="AC35" s="66"/>
+    </row>
+    <row r="36" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B36" s="6"/>
       <c r="C36" s="91"/>
       <c r="D36" s="91"/>
-      <c r="E36" s="95"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="38"/>
-      <c r="I36" s="44"/>
-      <c r="J36" s="40"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="44"/>
-      <c r="M36" s="40"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="38"/>
-      <c r="P36" s="40"/>
-      <c r="Q36" s="57"/>
+      <c r="E36" s="91"/>
+      <c r="F36" s="95"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="38"/>
+      <c r="J36" s="44"/>
+      <c r="K36" s="40"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="44"/>
+      <c r="N36" s="40"/>
+      <c r="O36" s="42"/>
+      <c r="P36" s="38"/>
+      <c r="Q36" s="40"/>
       <c r="R36" s="57"/>
       <c r="S36" s="57"/>
-      <c r="T36" s="40"/>
-      <c r="U36" s="54"/>
-      <c r="V36" s="44"/>
-      <c r="W36" s="40"/>
-      <c r="X36" s="57"/>
+      <c r="T36" s="57"/>
+      <c r="U36" s="40"/>
+      <c r="V36" s="54"/>
+      <c r="W36" s="44"/>
+      <c r="X36" s="40"/>
       <c r="Y36" s="57"/>
       <c r="Z36" s="57"/>
-      <c r="AA36" s="40"/>
-      <c r="AB36" s="66"/>
-    </row>
-    <row r="37" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA36" s="57"/>
+      <c r="AB36" s="40"/>
+      <c r="AC36" s="66"/>
+    </row>
+    <row r="37" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B37" s="6"/>
       <c r="C37" s="91"/>
       <c r="D37" s="91"/>
-      <c r="E37" s="95"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="44"/>
-      <c r="J37" s="40"/>
-      <c r="K37" s="42"/>
-      <c r="L37" s="44"/>
-      <c r="M37" s="40"/>
-      <c r="N37" s="42"/>
-      <c r="O37" s="38"/>
-      <c r="P37" s="40"/>
-      <c r="Q37" s="57"/>
+      <c r="E37" s="91"/>
+      <c r="F37" s="95"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="38"/>
+      <c r="J37" s="44"/>
+      <c r="K37" s="40"/>
+      <c r="L37" s="42"/>
+      <c r="M37" s="44"/>
+      <c r="N37" s="40"/>
+      <c r="O37" s="42"/>
+      <c r="P37" s="38"/>
+      <c r="Q37" s="40"/>
       <c r="R37" s="57"/>
       <c r="S37" s="57"/>
-      <c r="T37" s="40"/>
-      <c r="U37" s="54"/>
-      <c r="V37" s="44"/>
-      <c r="W37" s="40"/>
-      <c r="X37" s="57"/>
+      <c r="T37" s="57"/>
+      <c r="U37" s="40"/>
+      <c r="V37" s="54"/>
+      <c r="W37" s="44"/>
+      <c r="X37" s="40"/>
       <c r="Y37" s="57"/>
       <c r="Z37" s="57"/>
-      <c r="AA37" s="40"/>
-      <c r="AB37" s="66"/>
-    </row>
-    <row r="38" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA37" s="57"/>
+      <c r="AB37" s="40"/>
+      <c r="AC37" s="66"/>
+    </row>
+    <row r="38" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B38" s="6"/>
       <c r="C38" s="91"/>
       <c r="D38" s="91"/>
-      <c r="E38" s="95"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="44"/>
-      <c r="J38" s="40"/>
-      <c r="K38" s="42"/>
-      <c r="L38" s="44"/>
-      <c r="M38" s="40"/>
-      <c r="N38" s="42"/>
-      <c r="O38" s="38"/>
-      <c r="P38" s="40"/>
-      <c r="Q38" s="57"/>
+      <c r="E38" s="91"/>
+      <c r="F38" s="95"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="44"/>
+      <c r="K38" s="40"/>
+      <c r="L38" s="42"/>
+      <c r="M38" s="44"/>
+      <c r="N38" s="40"/>
+      <c r="O38" s="42"/>
+      <c r="P38" s="38"/>
+      <c r="Q38" s="40"/>
       <c r="R38" s="57"/>
       <c r="S38" s="57"/>
-      <c r="T38" s="40"/>
-      <c r="U38" s="54"/>
-      <c r="V38" s="44"/>
-      <c r="W38" s="40"/>
-      <c r="X38" s="57"/>
+      <c r="T38" s="57"/>
+      <c r="U38" s="40"/>
+      <c r="V38" s="54"/>
+      <c r="W38" s="44"/>
+      <c r="X38" s="40"/>
       <c r="Y38" s="57"/>
       <c r="Z38" s="57"/>
-      <c r="AA38" s="40"/>
-      <c r="AB38" s="66"/>
-    </row>
-    <row r="39" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA38" s="57"/>
+      <c r="AB38" s="40"/>
+      <c r="AC38" s="66"/>
+    </row>
+    <row r="39" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B39" s="6"/>
       <c r="C39" s="91"/>
       <c r="D39" s="91"/>
-      <c r="E39" s="95"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="40"/>
-      <c r="K39" s="42"/>
-      <c r="L39" s="44"/>
-      <c r="M39" s="40"/>
-      <c r="N39" s="42"/>
-      <c r="O39" s="38"/>
-      <c r="P39" s="40"/>
-      <c r="Q39" s="57"/>
+      <c r="E39" s="91"/>
+      <c r="F39" s="95"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="44"/>
+      <c r="K39" s="40"/>
+      <c r="L39" s="42"/>
+      <c r="M39" s="44"/>
+      <c r="N39" s="40"/>
+      <c r="O39" s="42"/>
+      <c r="P39" s="38"/>
+      <c r="Q39" s="40"/>
       <c r="R39" s="57"/>
       <c r="S39" s="57"/>
-      <c r="T39" s="40"/>
-      <c r="U39" s="54"/>
-      <c r="V39" s="44"/>
-      <c r="W39" s="40"/>
-      <c r="X39" s="57"/>
+      <c r="T39" s="57"/>
+      <c r="U39" s="40"/>
+      <c r="V39" s="54"/>
+      <c r="W39" s="44"/>
+      <c r="X39" s="40"/>
       <c r="Y39" s="57"/>
       <c r="Z39" s="57"/>
-      <c r="AA39" s="40"/>
-      <c r="AB39" s="66"/>
-    </row>
-    <row r="40" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA39" s="57"/>
+      <c r="AB39" s="40"/>
+      <c r="AC39" s="66"/>
+    </row>
+    <row r="40" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B40" s="6"/>
       <c r="C40" s="91"/>
       <c r="D40" s="91"/>
-      <c r="E40" s="95"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="38"/>
-      <c r="I40" s="44"/>
-      <c r="J40" s="40"/>
-      <c r="K40" s="42"/>
-      <c r="L40" s="44"/>
-      <c r="M40" s="40"/>
-      <c r="N40" s="42"/>
-      <c r="O40" s="38"/>
-      <c r="P40" s="40"/>
-      <c r="Q40" s="57"/>
+      <c r="E40" s="91"/>
+      <c r="F40" s="95"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="38"/>
+      <c r="J40" s="44"/>
+      <c r="K40" s="40"/>
+      <c r="L40" s="42"/>
+      <c r="M40" s="44"/>
+      <c r="N40" s="40"/>
+      <c r="O40" s="42"/>
+      <c r="P40" s="38"/>
+      <c r="Q40" s="40"/>
       <c r="R40" s="57"/>
       <c r="S40" s="57"/>
-      <c r="T40" s="40"/>
-      <c r="U40" s="54"/>
-      <c r="V40" s="44"/>
-      <c r="W40" s="40"/>
-      <c r="X40" s="57"/>
+      <c r="T40" s="57"/>
+      <c r="U40" s="40"/>
+      <c r="V40" s="54"/>
+      <c r="W40" s="44"/>
+      <c r="X40" s="40"/>
       <c r="Y40" s="57"/>
       <c r="Z40" s="57"/>
-      <c r="AA40" s="40"/>
-      <c r="AB40" s="66"/>
-    </row>
-    <row r="41" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA40" s="57"/>
+      <c r="AB40" s="40"/>
+      <c r="AC40" s="66"/>
+    </row>
+    <row r="41" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B41" s="6"/>
       <c r="C41" s="91"/>
       <c r="D41" s="91"/>
-      <c r="E41" s="95"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="44"/>
-      <c r="J41" s="40"/>
-      <c r="K41" s="42"/>
-      <c r="L41" s="44"/>
-      <c r="M41" s="40"/>
-      <c r="N41" s="42"/>
-      <c r="O41" s="38"/>
-      <c r="P41" s="40"/>
-      <c r="Q41" s="57"/>
+      <c r="E41" s="91"/>
+      <c r="F41" s="95"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="38"/>
+      <c r="J41" s="44"/>
+      <c r="K41" s="40"/>
+      <c r="L41" s="42"/>
+      <c r="M41" s="44"/>
+      <c r="N41" s="40"/>
+      <c r="O41" s="42"/>
+      <c r="P41" s="38"/>
+      <c r="Q41" s="40"/>
       <c r="R41" s="57"/>
       <c r="S41" s="57"/>
-      <c r="T41" s="40"/>
-      <c r="U41" s="54"/>
-      <c r="V41" s="44"/>
-      <c r="W41" s="40"/>
-      <c r="X41" s="57"/>
+      <c r="T41" s="57"/>
+      <c r="U41" s="40"/>
+      <c r="V41" s="54"/>
+      <c r="W41" s="44"/>
+      <c r="X41" s="40"/>
       <c r="Y41" s="57"/>
       <c r="Z41" s="57"/>
-      <c r="AA41" s="40"/>
-      <c r="AB41" s="66"/>
-    </row>
-    <row r="42" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA41" s="57"/>
+      <c r="AB41" s="40"/>
+      <c r="AC41" s="66"/>
+    </row>
+    <row r="42" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B42" s="6"/>
       <c r="C42" s="91"/>
       <c r="D42" s="91"/>
-      <c r="E42" s="95"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="38"/>
-      <c r="I42" s="44"/>
-      <c r="J42" s="40"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="44"/>
-      <c r="M42" s="40"/>
-      <c r="N42" s="42"/>
-      <c r="O42" s="38"/>
-      <c r="P42" s="40"/>
-      <c r="Q42" s="57"/>
+      <c r="E42" s="91"/>
+      <c r="F42" s="95"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="38"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="40"/>
+      <c r="L42" s="42"/>
+      <c r="M42" s="44"/>
+      <c r="N42" s="40"/>
+      <c r="O42" s="42"/>
+      <c r="P42" s="38"/>
+      <c r="Q42" s="40"/>
       <c r="R42" s="57"/>
       <c r="S42" s="57"/>
-      <c r="T42" s="40"/>
-      <c r="U42" s="54"/>
-      <c r="V42" s="44"/>
-      <c r="W42" s="40"/>
-      <c r="X42" s="57"/>
+      <c r="T42" s="57"/>
+      <c r="U42" s="40"/>
+      <c r="V42" s="54"/>
+      <c r="W42" s="44"/>
+      <c r="X42" s="40"/>
       <c r="Y42" s="57"/>
       <c r="Z42" s="57"/>
-      <c r="AA42" s="40"/>
-      <c r="AB42" s="66"/>
-    </row>
-    <row r="43" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA42" s="57"/>
+      <c r="AB42" s="40"/>
+      <c r="AC42" s="66"/>
+    </row>
+    <row r="43" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B43" s="6"/>
       <c r="C43" s="91"/>
       <c r="D43" s="91"/>
-      <c r="E43" s="95"/>
-      <c r="F43" s="11"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="38"/>
-      <c r="I43" s="44"/>
-      <c r="J43" s="40"/>
-      <c r="K43" s="42"/>
-      <c r="L43" s="44"/>
-      <c r="M43" s="40"/>
-      <c r="N43" s="42"/>
-      <c r="O43" s="38"/>
-      <c r="P43" s="40"/>
-      <c r="Q43" s="57"/>
+      <c r="E43" s="91"/>
+      <c r="F43" s="95"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="38"/>
+      <c r="J43" s="44"/>
+      <c r="K43" s="40"/>
+      <c r="L43" s="42"/>
+      <c r="M43" s="44"/>
+      <c r="N43" s="40"/>
+      <c r="O43" s="42"/>
+      <c r="P43" s="38"/>
+      <c r="Q43" s="40"/>
       <c r="R43" s="57"/>
       <c r="S43" s="57"/>
-      <c r="T43" s="40"/>
-      <c r="U43" s="54"/>
-      <c r="V43" s="44"/>
-      <c r="W43" s="40"/>
-      <c r="X43" s="57"/>
+      <c r="T43" s="57"/>
+      <c r="U43" s="40"/>
+      <c r="V43" s="54"/>
+      <c r="W43" s="44"/>
+      <c r="X43" s="40"/>
       <c r="Y43" s="57"/>
       <c r="Z43" s="57"/>
-      <c r="AA43" s="40"/>
-      <c r="AB43" s="66"/>
-    </row>
-    <row r="44" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA43" s="57"/>
+      <c r="AB43" s="40"/>
+      <c r="AC43" s="66"/>
+    </row>
+    <row r="44" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B44" s="6"/>
       <c r="C44" s="91"/>
       <c r="D44" s="91"/>
-      <c r="E44" s="95"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="38"/>
-      <c r="I44" s="44"/>
-      <c r="J44" s="40"/>
-      <c r="K44" s="42"/>
-      <c r="L44" s="44"/>
-      <c r="M44" s="40"/>
-      <c r="N44" s="42"/>
-      <c r="O44" s="38"/>
-      <c r="P44" s="40"/>
-      <c r="Q44" s="57"/>
+      <c r="E44" s="91"/>
+      <c r="F44" s="95"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="38"/>
+      <c r="J44" s="44"/>
+      <c r="K44" s="40"/>
+      <c r="L44" s="42"/>
+      <c r="M44" s="44"/>
+      <c r="N44" s="40"/>
+      <c r="O44" s="42"/>
+      <c r="P44" s="38"/>
+      <c r="Q44" s="40"/>
       <c r="R44" s="57"/>
       <c r="S44" s="57"/>
-      <c r="T44" s="40"/>
-      <c r="U44" s="54"/>
-      <c r="V44" s="44"/>
-      <c r="W44" s="40"/>
-      <c r="X44" s="57"/>
+      <c r="T44" s="57"/>
+      <c r="U44" s="40"/>
+      <c r="V44" s="54"/>
+      <c r="W44" s="44"/>
+      <c r="X44" s="40"/>
       <c r="Y44" s="57"/>
       <c r="Z44" s="57"/>
-      <c r="AA44" s="40"/>
-      <c r="AB44" s="66"/>
-    </row>
-    <row r="45" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA44" s="57"/>
+      <c r="AB44" s="40"/>
+      <c r="AC44" s="66"/>
+    </row>
+    <row r="45" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B45" s="6"/>
       <c r="C45" s="91"/>
       <c r="D45" s="91"/>
-      <c r="E45" s="95"/>
-      <c r="F45" s="11"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="38"/>
-      <c r="I45" s="44"/>
-      <c r="J45" s="40"/>
-      <c r="K45" s="42"/>
-      <c r="L45" s="44"/>
-      <c r="M45" s="40"/>
-      <c r="N45" s="42"/>
-      <c r="O45" s="38"/>
-      <c r="P45" s="40"/>
-      <c r="Q45" s="57"/>
+      <c r="E45" s="91"/>
+      <c r="F45" s="95"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="9"/>
+      <c r="I45" s="38"/>
+      <c r="J45" s="44"/>
+      <c r="K45" s="40"/>
+      <c r="L45" s="42"/>
+      <c r="M45" s="44"/>
+      <c r="N45" s="40"/>
+      <c r="O45" s="42"/>
+      <c r="P45" s="38"/>
+      <c r="Q45" s="40"/>
       <c r="R45" s="57"/>
       <c r="S45" s="57"/>
-      <c r="T45" s="40"/>
-      <c r="U45" s="54"/>
-      <c r="V45" s="44"/>
-      <c r="W45" s="40"/>
-      <c r="X45" s="57"/>
+      <c r="T45" s="57"/>
+      <c r="U45" s="40"/>
+      <c r="V45" s="54"/>
+      <c r="W45" s="44"/>
+      <c r="X45" s="40"/>
       <c r="Y45" s="57"/>
       <c r="Z45" s="57"/>
-      <c r="AA45" s="40"/>
-      <c r="AB45" s="66"/>
-    </row>
-    <row r="46" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA45" s="57"/>
+      <c r="AB45" s="40"/>
+      <c r="AC45" s="66"/>
+    </row>
+    <row r="46" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B46" s="6"/>
       <c r="C46" s="91"/>
       <c r="D46" s="91"/>
-      <c r="E46" s="95"/>
-      <c r="F46" s="11"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="38"/>
-      <c r="I46" s="44"/>
-      <c r="J46" s="40"/>
-      <c r="K46" s="42"/>
-      <c r="L46" s="44"/>
-      <c r="M46" s="40"/>
-      <c r="N46" s="42"/>
-      <c r="O46" s="38"/>
-      <c r="P46" s="40"/>
-      <c r="Q46" s="57"/>
+      <c r="E46" s="91"/>
+      <c r="F46" s="95"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="38"/>
+      <c r="J46" s="44"/>
+      <c r="K46" s="40"/>
+      <c r="L46" s="42"/>
+      <c r="M46" s="44"/>
+      <c r="N46" s="40"/>
+      <c r="O46" s="42"/>
+      <c r="P46" s="38"/>
+      <c r="Q46" s="40"/>
       <c r="R46" s="57"/>
       <c r="S46" s="57"/>
-      <c r="T46" s="40"/>
-      <c r="U46" s="54"/>
-      <c r="V46" s="44"/>
-      <c r="W46" s="40"/>
-      <c r="X46" s="57"/>
+      <c r="T46" s="57"/>
+      <c r="U46" s="40"/>
+      <c r="V46" s="54"/>
+      <c r="W46" s="44"/>
+      <c r="X46" s="40"/>
       <c r="Y46" s="57"/>
       <c r="Z46" s="57"/>
-      <c r="AA46" s="40"/>
-      <c r="AB46" s="66"/>
-    </row>
-    <row r="47" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA46" s="57"/>
+      <c r="AB46" s="40"/>
+      <c r="AC46" s="66"/>
+    </row>
+    <row r="47" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B47" s="6"/>
       <c r="C47" s="91"/>
       <c r="D47" s="91"/>
-      <c r="E47" s="95"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="38"/>
-      <c r="I47" s="44"/>
-      <c r="J47" s="40"/>
-      <c r="K47" s="42"/>
-      <c r="L47" s="44"/>
-      <c r="M47" s="40"/>
-      <c r="N47" s="42"/>
-      <c r="O47" s="38"/>
-      <c r="P47" s="40"/>
-      <c r="Q47" s="57"/>
+      <c r="E47" s="91"/>
+      <c r="F47" s="95"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="38"/>
+      <c r="J47" s="44"/>
+      <c r="K47" s="40"/>
+      <c r="L47" s="42"/>
+      <c r="M47" s="44"/>
+      <c r="N47" s="40"/>
+      <c r="O47" s="42"/>
+      <c r="P47" s="38"/>
+      <c r="Q47" s="40"/>
       <c r="R47" s="57"/>
       <c r="S47" s="57"/>
-      <c r="T47" s="40"/>
-      <c r="U47" s="54"/>
-      <c r="V47" s="44"/>
-      <c r="W47" s="40"/>
-      <c r="X47" s="57"/>
+      <c r="T47" s="57"/>
+      <c r="U47" s="40"/>
+      <c r="V47" s="54"/>
+      <c r="W47" s="44"/>
+      <c r="X47" s="40"/>
       <c r="Y47" s="57"/>
       <c r="Z47" s="57"/>
-      <c r="AA47" s="40"/>
-      <c r="AB47" s="66"/>
-    </row>
-    <row r="48" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA47" s="57"/>
+      <c r="AB47" s="40"/>
+      <c r="AC47" s="66"/>
+    </row>
+    <row r="48" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B48" s="6"/>
       <c r="C48" s="91"/>
       <c r="D48" s="91"/>
-      <c r="E48" s="95"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="38"/>
-      <c r="I48" s="44"/>
-      <c r="J48" s="40"/>
-      <c r="K48" s="42"/>
-      <c r="L48" s="44"/>
-      <c r="M48" s="40"/>
-      <c r="N48" s="42"/>
-      <c r="O48" s="38"/>
-      <c r="P48" s="40"/>
-      <c r="Q48" s="57"/>
+      <c r="E48" s="91"/>
+      <c r="F48" s="95"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="9"/>
+      <c r="I48" s="38"/>
+      <c r="J48" s="44"/>
+      <c r="K48" s="40"/>
+      <c r="L48" s="42"/>
+      <c r="M48" s="44"/>
+      <c r="N48" s="40"/>
+      <c r="O48" s="42"/>
+      <c r="P48" s="38"/>
+      <c r="Q48" s="40"/>
       <c r="R48" s="57"/>
       <c r="S48" s="57"/>
-      <c r="T48" s="40"/>
-      <c r="U48" s="54"/>
-      <c r="V48" s="44"/>
-      <c r="W48" s="40"/>
-      <c r="X48" s="57"/>
+      <c r="T48" s="57"/>
+      <c r="U48" s="40"/>
+      <c r="V48" s="54"/>
+      <c r="W48" s="44"/>
+      <c r="X48" s="40"/>
       <c r="Y48" s="57"/>
       <c r="Z48" s="57"/>
-      <c r="AA48" s="40"/>
-      <c r="AB48" s="66"/>
-    </row>
-    <row r="49" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA48" s="57"/>
+      <c r="AB48" s="40"/>
+      <c r="AC48" s="66"/>
+    </row>
+    <row r="49" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B49" s="6"/>
       <c r="C49" s="91"/>
       <c r="D49" s="91"/>
-      <c r="E49" s="95"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="9"/>
-      <c r="H49" s="38"/>
-      <c r="I49" s="44"/>
-      <c r="J49" s="40"/>
-      <c r="K49" s="42"/>
-      <c r="L49" s="44"/>
-      <c r="M49" s="40"/>
-      <c r="N49" s="42"/>
-      <c r="O49" s="38"/>
-      <c r="P49" s="40"/>
-      <c r="Q49" s="57"/>
+      <c r="E49" s="91"/>
+      <c r="F49" s="95"/>
+      <c r="G49" s="11"/>
+      <c r="H49" s="9"/>
+      <c r="I49" s="38"/>
+      <c r="J49" s="44"/>
+      <c r="K49" s="40"/>
+      <c r="L49" s="42"/>
+      <c r="M49" s="44"/>
+      <c r="N49" s="40"/>
+      <c r="O49" s="42"/>
+      <c r="P49" s="38"/>
+      <c r="Q49" s="40"/>
       <c r="R49" s="57"/>
       <c r="S49" s="57"/>
-      <c r="T49" s="40"/>
-      <c r="U49" s="54"/>
-      <c r="V49" s="44"/>
-      <c r="W49" s="40"/>
-      <c r="X49" s="57"/>
+      <c r="T49" s="57"/>
+      <c r="U49" s="40"/>
+      <c r="V49" s="54"/>
+      <c r="W49" s="44"/>
+      <c r="X49" s="40"/>
       <c r="Y49" s="57"/>
       <c r="Z49" s="57"/>
-      <c r="AA49" s="40"/>
-      <c r="AB49" s="66"/>
-    </row>
-    <row r="50" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA49" s="57"/>
+      <c r="AB49" s="40"/>
+      <c r="AC49" s="66"/>
+    </row>
+    <row r="50" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B50" s="6"/>
       <c r="C50" s="91"/>
       <c r="D50" s="91"/>
-      <c r="E50" s="95"/>
-      <c r="F50" s="11"/>
-      <c r="G50" s="9"/>
-      <c r="H50" s="38"/>
-      <c r="I50" s="44"/>
-      <c r="J50" s="40"/>
-      <c r="K50" s="42"/>
-      <c r="L50" s="44"/>
-      <c r="M50" s="40"/>
-      <c r="N50" s="42"/>
-      <c r="O50" s="38"/>
-      <c r="P50" s="40"/>
-      <c r="Q50" s="57"/>
+      <c r="E50" s="91"/>
+      <c r="F50" s="95"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="9"/>
+      <c r="I50" s="38"/>
+      <c r="J50" s="44"/>
+      <c r="K50" s="40"/>
+      <c r="L50" s="42"/>
+      <c r="M50" s="44"/>
+      <c r="N50" s="40"/>
+      <c r="O50" s="42"/>
+      <c r="P50" s="38"/>
+      <c r="Q50" s="40"/>
       <c r="R50" s="57"/>
       <c r="S50" s="57"/>
-      <c r="T50" s="40"/>
-      <c r="U50" s="54"/>
-      <c r="V50" s="44"/>
-      <c r="W50" s="40"/>
-      <c r="X50" s="57"/>
+      <c r="T50" s="57"/>
+      <c r="U50" s="40"/>
+      <c r="V50" s="54"/>
+      <c r="W50" s="44"/>
+      <c r="X50" s="40"/>
       <c r="Y50" s="57"/>
       <c r="Z50" s="57"/>
-      <c r="AA50" s="40"/>
-      <c r="AB50" s="66"/>
-    </row>
-    <row r="51" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA50" s="57"/>
+      <c r="AB50" s="40"/>
+      <c r="AC50" s="66"/>
+    </row>
+    <row r="51" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B51" s="6"/>
       <c r="C51" s="91"/>
       <c r="D51" s="91"/>
-      <c r="E51" s="95"/>
-      <c r="F51" s="11"/>
-      <c r="G51" s="9"/>
-      <c r="H51" s="38"/>
-      <c r="I51" s="44"/>
-      <c r="J51" s="40"/>
-      <c r="K51" s="42"/>
-      <c r="L51" s="44"/>
-      <c r="M51" s="40"/>
-      <c r="N51" s="42"/>
-      <c r="O51" s="38"/>
-      <c r="P51" s="40"/>
-      <c r="Q51" s="57"/>
+      <c r="E51" s="91"/>
+      <c r="F51" s="95"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="38"/>
+      <c r="J51" s="44"/>
+      <c r="K51" s="40"/>
+      <c r="L51" s="42"/>
+      <c r="M51" s="44"/>
+      <c r="N51" s="40"/>
+      <c r="O51" s="42"/>
+      <c r="P51" s="38"/>
+      <c r="Q51" s="40"/>
       <c r="R51" s="57"/>
       <c r="S51" s="57"/>
-      <c r="T51" s="40"/>
-      <c r="U51" s="54"/>
-      <c r="V51" s="44"/>
-      <c r="W51" s="40"/>
-      <c r="X51" s="57"/>
+      <c r="T51" s="57"/>
+      <c r="U51" s="40"/>
+      <c r="V51" s="54"/>
+      <c r="W51" s="44"/>
+      <c r="X51" s="40"/>
       <c r="Y51" s="57"/>
       <c r="Z51" s="57"/>
-      <c r="AA51" s="40"/>
-      <c r="AB51" s="66"/>
-    </row>
-    <row r="52" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA51" s="57"/>
+      <c r="AB51" s="40"/>
+      <c r="AC51" s="66"/>
+    </row>
+    <row r="52" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B52" s="6"/>
       <c r="C52" s="91"/>
       <c r="D52" s="91"/>
-      <c r="E52" s="95"/>
-      <c r="F52" s="11"/>
-      <c r="G52" s="9"/>
-      <c r="H52" s="38"/>
-      <c r="I52" s="44"/>
-      <c r="J52" s="40"/>
-      <c r="K52" s="42"/>
-      <c r="L52" s="44"/>
-      <c r="M52" s="40"/>
-      <c r="N52" s="42"/>
-      <c r="O52" s="38"/>
-      <c r="P52" s="40"/>
-      <c r="Q52" s="57"/>
+      <c r="E52" s="91"/>
+      <c r="F52" s="95"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="9"/>
+      <c r="I52" s="38"/>
+      <c r="J52" s="44"/>
+      <c r="K52" s="40"/>
+      <c r="L52" s="42"/>
+      <c r="M52" s="44"/>
+      <c r="N52" s="40"/>
+      <c r="O52" s="42"/>
+      <c r="P52" s="38"/>
+      <c r="Q52" s="40"/>
       <c r="R52" s="57"/>
       <c r="S52" s="57"/>
-      <c r="T52" s="40"/>
-      <c r="U52" s="54"/>
-      <c r="V52" s="44"/>
-      <c r="W52" s="40"/>
-      <c r="X52" s="57"/>
+      <c r="T52" s="57"/>
+      <c r="U52" s="40"/>
+      <c r="V52" s="54"/>
+      <c r="W52" s="44"/>
+      <c r="X52" s="40"/>
       <c r="Y52" s="57"/>
       <c r="Z52" s="57"/>
-      <c r="AA52" s="40"/>
-      <c r="AB52" s="66"/>
-    </row>
-    <row r="53" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA52" s="57"/>
+      <c r="AB52" s="40"/>
+      <c r="AC52" s="66"/>
+    </row>
+    <row r="53" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B53" s="6"/>
       <c r="C53" s="91"/>
       <c r="D53" s="91"/>
-      <c r="E53" s="95"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="9"/>
-      <c r="H53" s="38"/>
-      <c r="I53" s="44"/>
-      <c r="J53" s="40"/>
-      <c r="K53" s="42"/>
-      <c r="L53" s="44"/>
-      <c r="M53" s="40"/>
-      <c r="N53" s="42"/>
-      <c r="O53" s="38"/>
-      <c r="P53" s="40"/>
-      <c r="Q53" s="57"/>
+      <c r="E53" s="91"/>
+      <c r="F53" s="95"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="38"/>
+      <c r="J53" s="44"/>
+      <c r="K53" s="40"/>
+      <c r="L53" s="42"/>
+      <c r="M53" s="44"/>
+      <c r="N53" s="40"/>
+      <c r="O53" s="42"/>
+      <c r="P53" s="38"/>
+      <c r="Q53" s="40"/>
       <c r="R53" s="57"/>
       <c r="S53" s="57"/>
-      <c r="T53" s="40"/>
-      <c r="U53" s="54"/>
-      <c r="V53" s="44"/>
-      <c r="W53" s="40"/>
-      <c r="X53" s="57"/>
+      <c r="T53" s="57"/>
+      <c r="U53" s="40"/>
+      <c r="V53" s="54"/>
+      <c r="W53" s="44"/>
+      <c r="X53" s="40"/>
       <c r="Y53" s="57"/>
       <c r="Z53" s="57"/>
-      <c r="AA53" s="40"/>
-      <c r="AB53" s="66"/>
-    </row>
-    <row r="54" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA53" s="57"/>
+      <c r="AB53" s="40"/>
+      <c r="AC53" s="66"/>
+    </row>
+    <row r="54" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B54" s="6"/>
       <c r="C54" s="91"/>
       <c r="D54" s="91"/>
-      <c r="E54" s="95"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="9"/>
-      <c r="H54" s="38"/>
-      <c r="I54" s="44"/>
-      <c r="J54" s="40"/>
-      <c r="K54" s="42"/>
-      <c r="L54" s="44"/>
-      <c r="M54" s="40"/>
-      <c r="N54" s="42"/>
-      <c r="O54" s="38"/>
-      <c r="P54" s="40"/>
-      <c r="Q54" s="57"/>
+      <c r="E54" s="91"/>
+      <c r="F54" s="95"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="38"/>
+      <c r="J54" s="44"/>
+      <c r="K54" s="40"/>
+      <c r="L54" s="42"/>
+      <c r="M54" s="44"/>
+      <c r="N54" s="40"/>
+      <c r="O54" s="42"/>
+      <c r="P54" s="38"/>
+      <c r="Q54" s="40"/>
       <c r="R54" s="57"/>
       <c r="S54" s="57"/>
-      <c r="T54" s="40"/>
-      <c r="U54" s="54"/>
-      <c r="V54" s="44"/>
-      <c r="W54" s="40"/>
-      <c r="X54" s="57"/>
+      <c r="T54" s="57"/>
+      <c r="U54" s="40"/>
+      <c r="V54" s="54"/>
+      <c r="W54" s="44"/>
+      <c r="X54" s="40"/>
       <c r="Y54" s="57"/>
       <c r="Z54" s="57"/>
-      <c r="AA54" s="40"/>
-      <c r="AB54" s="66"/>
-    </row>
-    <row r="55" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA54" s="57"/>
+      <c r="AB54" s="40"/>
+      <c r="AC54" s="66"/>
+    </row>
+    <row r="55" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B55" s="6"/>
       <c r="C55" s="91"/>
       <c r="D55" s="91"/>
-      <c r="E55" s="95"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="9"/>
-      <c r="H55" s="38"/>
-      <c r="I55" s="44"/>
-      <c r="J55" s="40"/>
-      <c r="K55" s="42"/>
-      <c r="L55" s="44"/>
-      <c r="M55" s="40"/>
-      <c r="N55" s="42"/>
-      <c r="O55" s="38"/>
-      <c r="P55" s="40"/>
-      <c r="Q55" s="57"/>
+      <c r="E55" s="91"/>
+      <c r="F55" s="95"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="9"/>
+      <c r="I55" s="38"/>
+      <c r="J55" s="44"/>
+      <c r="K55" s="40"/>
+      <c r="L55" s="42"/>
+      <c r="M55" s="44"/>
+      <c r="N55" s="40"/>
+      <c r="O55" s="42"/>
+      <c r="P55" s="38"/>
+      <c r="Q55" s="40"/>
       <c r="R55" s="57"/>
       <c r="S55" s="57"/>
-      <c r="T55" s="40"/>
-      <c r="U55" s="54"/>
-      <c r="V55" s="44"/>
-      <c r="W55" s="40"/>
-      <c r="X55" s="57"/>
+      <c r="T55" s="57"/>
+      <c r="U55" s="40"/>
+      <c r="V55" s="54"/>
+      <c r="W55" s="44"/>
+      <c r="X55" s="40"/>
       <c r="Y55" s="57"/>
       <c r="Z55" s="57"/>
-      <c r="AA55" s="40"/>
-      <c r="AB55" s="66"/>
-    </row>
-    <row r="56" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA55" s="57"/>
+      <c r="AB55" s="40"/>
+      <c r="AC55" s="66"/>
+    </row>
+    <row r="56" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B56" s="6"/>
       <c r="C56" s="91"/>
       <c r="D56" s="91"/>
-      <c r="E56" s="95"/>
-      <c r="F56" s="11"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="38"/>
-      <c r="I56" s="44"/>
-      <c r="J56" s="40"/>
-      <c r="K56" s="42"/>
-      <c r="L56" s="44"/>
-      <c r="M56" s="40"/>
-      <c r="N56" s="42"/>
-      <c r="O56" s="38"/>
-      <c r="P56" s="40"/>
-      <c r="Q56" s="57"/>
+      <c r="E56" s="91"/>
+      <c r="F56" s="95"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="38"/>
+      <c r="J56" s="44"/>
+      <c r="K56" s="40"/>
+      <c r="L56" s="42"/>
+      <c r="M56" s="44"/>
+      <c r="N56" s="40"/>
+      <c r="O56" s="42"/>
+      <c r="P56" s="38"/>
+      <c r="Q56" s="40"/>
       <c r="R56" s="57"/>
       <c r="S56" s="57"/>
-      <c r="T56" s="40"/>
-      <c r="U56" s="54"/>
-      <c r="V56" s="44"/>
-      <c r="W56" s="40"/>
-      <c r="X56" s="57"/>
+      <c r="T56" s="57"/>
+      <c r="U56" s="40"/>
+      <c r="V56" s="54"/>
+      <c r="W56" s="44"/>
+      <c r="X56" s="40"/>
       <c r="Y56" s="57"/>
       <c r="Z56" s="57"/>
-      <c r="AA56" s="40"/>
-      <c r="AB56" s="66"/>
-    </row>
-    <row r="57" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="AA56" s="57"/>
+      <c r="AB56" s="40"/>
+      <c r="AC56" s="66"/>
+    </row>
+    <row r="57" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B57" s="6"/>
       <c r="C57" s="91"/>
       <c r="D57" s="91"/>
-      <c r="E57" s="95"/>
-      <c r="F57" s="11"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="38"/>
-      <c r="I57" s="44"/>
-      <c r="J57" s="40"/>
-      <c r="K57" s="42"/>
-      <c r="L57" s="44"/>
-      <c r="M57" s="40"/>
-      <c r="N57" s="42"/>
-      <c r="O57" s="38"/>
-      <c r="P57" s="40"/>
-      <c r="Q57" s="57"/>
+      <c r="E57" s="91"/>
+      <c r="F57" s="95"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="9"/>
+      <c r="I57" s="38"/>
+      <c r="J57" s="44"/>
+      <c r="K57" s="40"/>
+      <c r="L57" s="42"/>
+      <c r="M57" s="44"/>
+      <c r="N57" s="40"/>
+      <c r="O57" s="42"/>
+      <c r="P57" s="38"/>
+      <c r="Q57" s="40"/>
       <c r="R57" s="57"/>
       <c r="S57" s="57"/>
-      <c r="T57" s="40"/>
-      <c r="U57" s="54"/>
-      <c r="V57" s="44"/>
-      <c r="W57" s="40"/>
-      <c r="X57" s="57"/>
+      <c r="T57" s="57"/>
+      <c r="U57" s="40"/>
+      <c r="V57" s="54"/>
+      <c r="W57" s="44"/>
+      <c r="X57" s="40"/>
       <c r="Y57" s="57"/>
       <c r="Z57" s="57"/>
-      <c r="AA57" s="40"/>
-      <c r="AB57" s="66"/>
+      <c r="AA57" s="57"/>
+      <c r="AB57" s="40"/>
+      <c r="AC57" s="66"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="XoJ5qKY8Y7diJeHOoqSg7/iXi7jVb2oZrNE3shpeeCqp4ZpWVDoC4maZ75Vu8I/xZdIwwFAlwW1C84unNxDyDg==" saltValue="B9Z2aag2RkRnYzQWHF1+rg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="trgYi39t6fkCckSxkO8ZwXGlCQRhjZHMePnMXMYXtAGGLXyMG1Lkz1Rz0OOcPaF2bKZ5ok0xhVRZ+jSGeL2ECg==" saltValue="xeSM1lhKUaExWmzVvHsbag==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="7">
-    <mergeCell ref="AD3:DY3"/>
-    <mergeCell ref="B2:AB3"/>
-    <mergeCell ref="B4:G6"/>
-    <mergeCell ref="H4:K6"/>
-    <mergeCell ref="L4:N6"/>
-    <mergeCell ref="O4:U6"/>
-    <mergeCell ref="V4:AB6"/>
+    <mergeCell ref="AE3:DZ3"/>
+    <mergeCell ref="B2:AC3"/>
+    <mergeCell ref="I4:L6"/>
+    <mergeCell ref="M4:O6"/>
+    <mergeCell ref="P4:V6"/>
+    <mergeCell ref="W4:AC6"/>
+    <mergeCell ref="B4:H6"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:AB1048576">
+  <conditionalFormatting sqref="B8:AC1048576">
     <cfRule type="expression" dxfId="1" priority="3">
       <formula>B8=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AD8:DY1048576">
+  <conditionalFormatting sqref="AE8:DZ1048576">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AD8=""</formula>
+      <formula>AE8=""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC4:AC7 L7 K7 B7 C7 D7 E7 F7 G7 H7 I7 J7 N7 M7" xr:uid="{86B40B65-30E0-465F-9E4E-BDD2D0A3ECB3}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD4:AD7 M7 L7 B7 N7 E7 C7 G7 H7 I7 J7 K7 O7 F7 D7" xr:uid="{86B40B65-30E0-465F-9E4E-BDD2D0A3ECB3}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="K7" r:id="rId1" location="FOBbuoyActivityTypes" xr:uid="{959EF245-C0B1-440F-9064-76CBE53740AB}"/>
-    <hyperlink ref="M7" r:id="rId2" location="FOBtypes" xr:uid="{0D9BDFCB-0E93-45FA-A9F8-2F2F4961FF03}"/>
-    <hyperlink ref="N7" r:id="rId3" location="FOBactivityTypes" xr:uid="{3C4B7339-15DC-4AE3-BA6F-6F6FE197BAF1}"/>
-    <hyperlink ref="AC6" r:id="rId4" location="raisings" xr:uid="{A80A0B5F-91B5-4F24-82CA-F4ED55F31384}"/>
-    <hyperlink ref="AC7" r:id="rId5" location="catchUnits" xr:uid="{CB8E1D12-F8A8-404C-8F09-27506E824907}"/>
-    <hyperlink ref="AC5" r:id="rId6" location="typesOfFate" xr:uid="{429FA315-D35E-430B-B16F-AFFF65DCB96E}"/>
-    <hyperlink ref="AC4" r:id="rId7" location="allSpecies" xr:uid="{ECADD488-F51B-467A-8AE5-D0932455B163}"/>
+    <hyperlink ref="L7" r:id="rId1" location="FOBbuoyActivityTypes" xr:uid="{959EF245-C0B1-440F-9064-76CBE53740AB}"/>
+    <hyperlink ref="N7" r:id="rId2" location="FOBtypes" xr:uid="{0D9BDFCB-0E93-45FA-A9F8-2F2F4961FF03}"/>
+    <hyperlink ref="O7" r:id="rId3" location="FOBactivityTypes" xr:uid="{3C4B7339-15DC-4AE3-BA6F-6F6FE197BAF1}"/>
+    <hyperlink ref="AD6" r:id="rId4" location="raisings" xr:uid="{A80A0B5F-91B5-4F24-82CA-F4ED55F31384}"/>
+    <hyperlink ref="AD7" r:id="rId5" location="catchUnits" xr:uid="{CB8E1D12-F8A8-404C-8F09-27506E824907}"/>
+    <hyperlink ref="AD5" r:id="rId6" location="typesOfFate" xr:uid="{429FA315-D35E-430B-B16F-AFFF65DCB96E}"/>
+    <hyperlink ref="AD4" r:id="rId7" location="allSpecies" xr:uid="{ECADD488-F51B-467A-8AE5-D0932455B163}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>

</xml_diff>